<commit_message>
Leads: 2026-09-13 13:13 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L129"/>
+  <dimension ref="A1:L133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7948,6 +7948,238 @@
         </is>
       </c>
     </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Air Conditioning Repair Houston, TX</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>ultimatecomfortac.com</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>https://www.ultimatecomfortac.com/ac-repair</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>office@ultimatecomfortac.com</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>(713) 359-9293</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Houston TX</t>
+        </is>
+      </c>
+      <c r="I130" t="n">
+        <v>100</v>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>air conditioning repair Houston TX</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Just Fix It Air Conditioning &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>justfixittoday.com</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>https://justfixittoday.com/air-conditioning/ac-repair/</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>noreply@justfixittoday.com</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>281-617-2231</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Houston TX</t>
+        </is>
+      </c>
+      <c r="I131" t="n">
+        <v>90</v>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>air conditioning repair Houston TX</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Air Tech of Houston</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>airtechofhouston.com</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>https://www.airtechofhouston.com/air-conditioning/ac-repair/</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Air Tech</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>service@airtechofhouston.com</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>(832) 699-4685</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Houston TX</t>
+        </is>
+      </c>
+      <c r="I132" t="n">
+        <v>90</v>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>air conditioning repair Houston TX</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Ray's Clearflow Plumbing NY</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>rcfpny.com</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>https://rcfpny.com/services/heat-pumps/</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Rays Clearflow</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>info@rcfpny.com</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>(518) 502-6128</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>Schenectady NY</t>
+        </is>
+      </c>
+      <c r="I133" t="n">
+        <v>90</v>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>heat pump installation Schenectady NY</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 13:16 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L133"/>
+  <dimension ref="A1:L135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7969,7 +7969,6 @@
           <t>https://www.ultimatecomfortac.com/ac-repair</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr">
         <is>
           <t>office@ultimatecomfortac.com</t>
@@ -8025,7 +8024,6 @@
           <t>https://justfixittoday.com/air-conditioning/ac-repair/</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr">
         <is>
           <t>noreply@justfixittoday.com</t>
@@ -8175,6 +8173,118 @@
         </is>
       </c>
       <c r="L133" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>OnlyHVACLLC</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>onlyhvacswfl.com</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>https://www.onlyhvacswfl.com/</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>example@mysite.com</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>239-428-4090</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Naples FL</t>
+        </is>
+      </c>
+      <c r="I134" t="n">
+        <v>96</v>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>HVAC contractor Naples FL</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>HVAC Contractor – Naples, FL – Mercury Rising HVAC Inc.</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>mercuryrisinghvac.com</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>https://www.mercuryrisinghvac.com/</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>ralph@mercuryrisinghvac.com</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>(239) 348-9927</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Naples FL</t>
+        </is>
+      </c>
+      <c r="I135" t="n">
+        <v>88</v>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>HVAC contractor Naples FL</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 13:18 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L135"/>
+  <dimension ref="A1:L140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8199,7 +8199,6 @@
           <t>https://www.onlyhvacswfl.com/</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr">
         <is>
           <t>example@mysite.com</t>
@@ -8255,7 +8254,6 @@
           <t>https://www.mercuryrisinghvac.com/</t>
         </is>
       </c>
-      <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr">
         <is>
           <t>ralph@mercuryrisinghvac.com</t>
@@ -8285,6 +8283,290 @@
         </is>
       </c>
       <c r="L135" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Quality Comfort Services, Inc.</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>qcshvac.com</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>https://qcshvac.com/residential-hvac/air-conditioning</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>kgreen@qcshvac.com</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>(919) 646-3296</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Raleigh NC</t>
+        </is>
+      </c>
+      <c r="I136" t="n">
+        <v>100</v>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>air conditioning repair Raleigh NC</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Expert Plumbing &amp; Heating Services | Sun Plumbing and Heating | Casper, Glenrock</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>sunplumbingandheatingllc.com</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>https://www.sunplumbingandheatingllc.com/</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>robertaplanalp@gmail.com</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>(307) 267-7959</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Casper WY</t>
+        </is>
+      </c>
+      <c r="I137" t="n">
+        <v>98</v>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>plumbing company Casper WY</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Cool Change NC</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>coolchangenc.com</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>https://www.coolchangenc.com/</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>yourinfo@fixingyourhvac.com</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>919-457-2494</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Raleigh NC</t>
+        </is>
+      </c>
+      <c r="I138" t="n">
+        <v>90</v>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>air conditioning repair Raleigh NC</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Lavoie Heating Service - Residential and Commercial HVAC Services</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>lavoieheatingservice.com</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>https://lavoieheatingservice.com/worcester/</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Central Massachusetts</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>info@lavoieheatingservice.com</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>508-791-5840</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Worcester MA</t>
+        </is>
+      </c>
+      <c r="I139" t="n">
+        <v>90</v>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>heating and cooling company Worcester MA</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Casper Plumbing</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>casperplumbing.com</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>https://www.casperplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>infocasperplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>307-441-4444</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Casper WY</t>
+        </is>
+      </c>
+      <c r="I140" t="n">
+        <v>70</v>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>plumbing company Casper WY</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 13:19 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L140"/>
+  <dimension ref="A1:L143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8309,7 +8309,6 @@
           <t>https://qcshvac.com/residential-hvac/air-conditioning</t>
         </is>
       </c>
-      <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr">
         <is>
           <t>kgreen@qcshvac.com</t>
@@ -8365,7 +8364,6 @@
           <t>https://www.sunplumbingandheatingllc.com/</t>
         </is>
       </c>
-      <c r="E137" t="inlineStr"/>
       <c r="F137" t="inlineStr">
         <is>
           <t>robertaplanalp@gmail.com</t>
@@ -8421,7 +8419,6 @@
           <t>https://www.coolchangenc.com/</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr">
         <is>
           <t>yourinfo@fixingyourhvac.com</t>
@@ -8537,7 +8534,6 @@
           <t>https://www.casperplumbing.com/</t>
         </is>
       </c>
-      <c r="E140" t="inlineStr"/>
       <c r="F140" t="inlineStr">
         <is>
           <t>infocasperplumbing@gmail.com</t>
@@ -8567,6 +8563,178 @@
         </is>
       </c>
       <c r="L140" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>OpenBox Roofing</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>openboxroofing.com</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>https://www.openboxroofing.com/locations/carmel/</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Megan Hughes</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>info@openboxroofing.com</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>(317) 619-9001</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Carmel IN</t>
+        </is>
+      </c>
+      <c r="I141" t="n">
+        <v>100</v>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>residential roofing company Carmel IN</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Arms Ac &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>armsac.com</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>https://armsac.com/services/heat-pumps-in-fresno-ca/</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>membership@armsac.com</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>209-357-8199</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Fresno CA</t>
+        </is>
+      </c>
+      <c r="I142" t="n">
+        <v>100</v>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>heat pump installation Fresno CA</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>AC Repair in Brownsville</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>acrepairinbrownsville.com</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>https://acrepairinbrownsville.com/</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>info@acrepairinbrownsville.com</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>956 670 8899</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Brownsville TX</t>
+        </is>
+      </c>
+      <c r="I143" t="n">
+        <v>88</v>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>air conditioning repair Brownsville TX</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 13:21 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L143"/>
+  <dimension ref="A1:L145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8649,7 +8649,6 @@
           <t>https://armsac.com/services/heat-pumps-in-fresno-ca/</t>
         </is>
       </c>
-      <c r="E142" t="inlineStr"/>
       <c r="F142" t="inlineStr">
         <is>
           <t>membership@armsac.com</t>
@@ -8705,7 +8704,6 @@
           <t>https://acrepairinbrownsville.com/</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr"/>
       <c r="F143" t="inlineStr">
         <is>
           <t>info@acrepairinbrownsville.com</t>
@@ -8735,6 +8733,126 @@
         </is>
       </c>
       <c r="L143" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Water Heater Repair &amp; Replacement in Aberdeen, SD</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>aberdeen-sd.winterplumbingandhvac.com</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>https://aberdeen-sd.winterplumbingandhvac.com/water-heater-repair-and-replacement/</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Nicole Plumbing</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>contact@winterplumbingandhvac.com</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>(855) 804-9142</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="I144" t="n">
+        <v>90</v>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>water heater repair Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>CoolBest AC Repair Pros</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>coolbestacrepair.pro</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>https://coolbestacrepair.pro/</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Team The</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>info@coolbestacrepair.pro</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>(812) 441-6186</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Bloomington IN</t>
+        </is>
+      </c>
+      <c r="I145" t="n">
+        <v>84</v>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>air conditioning repair Bloomington IN</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 13:22 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L145"/>
+  <dimension ref="A1:L152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8858,6 +8858,418 @@
         </is>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Brian Wear Plumbing</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>brianwearplumbing.com</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>https://brianwearplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>info@brianwearplumbing.com</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>573-303-5124</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Columbia MO</t>
+        </is>
+      </c>
+      <c r="I146" t="n">
+        <v>100</v>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>plumber Columbia MO</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Metal Roof Installation | High Point, NC</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>wmroofingpros.com</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>https://www.wmroofingpros.com/metal-roof-installation</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Decades Metal</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>shanebyerly@gmail.com</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>(336) 223-6765</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>High Point NC</t>
+        </is>
+      </c>
+      <c r="I147" t="n">
+        <v>100</v>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>metal roofing contractor High Point NC</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>www.excelroofingsolutions.com</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>excelroofingsolutions.com</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>https://excelroofingsolutions.com/service-areas/high-point/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>info@excelroofingsolutions.com</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>(336) 221-4121</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>High Point NC</t>
+        </is>
+      </c>
+      <c r="I148" t="n">
+        <v>100</v>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>metal roofing contractor High Point NC</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>College Station Roofing Company | Trophy Exteriors</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>trophyexteriors.com</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>https://www.trophyexteriors.com/college-station/</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>College Station</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>office@trophyexteriors.com</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>(979) 217-2748</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>College Station TX</t>
+        </is>
+      </c>
+      <c r="I149" t="n">
+        <v>100</v>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>roof replacement College Station TX</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Port St Lucie Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>portsaintlucieairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>https://portsaintlucieairconditioning.com/</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>email@portsaintlucieairconditioning.com</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>800-961-6480</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Port St Lucie FL</t>
+        </is>
+      </c>
+      <c r="I150" t="n">
+        <v>100</v>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>air conditioning repair Port St Lucie FL</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Residential Metal Roofing High Point NC | Licensed GC | B&amp;D Roofing</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>bndroofing.net</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>https://www.bndroofing.net/residential-roofing-high-point-nc/residential-metal-roofing</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Roofing Solutions</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>donna.frey@bndroofing.net</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>(336) 899-1985</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>High Point NC</t>
+        </is>
+      </c>
+      <c r="I151" t="n">
+        <v>90</v>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>metal roofing contractor High Point NC</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>newmanairconditioning.com</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>newmanairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>https://newmanairconditioning.com/ac-repair-port-st-lucie-fl/</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>What Our</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>khatodiasahil3@gmail.com</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>(863) 862-9924</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>Port St Lucie FL</t>
+        </is>
+      </c>
+      <c r="I152" t="n">
+        <v>90</v>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>air conditioning repair Port St Lucie FL</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 13:24 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L152"/>
+  <dimension ref="A1:L154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8999,7 +8999,6 @@
           <t>https://excelroofingsolutions.com/service-areas/high-point/metal-roofing/</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr"/>
       <c r="F148" t="inlineStr">
         <is>
           <t>info@excelroofingsolutions.com</t>
@@ -9115,7 +9114,6 @@
           <t>https://portsaintlucieairconditioning.com/</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr">
         <is>
           <t>email@portsaintlucieairconditioning.com</t>
@@ -9265,6 +9263,118 @@
         </is>
       </c>
       <c r="L152" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Total Comfort Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>totallycomfortable.com</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>https://totallycomfortable.com/furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr"/>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>heatingcoolingca@gmail.com</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>559-549-7227</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Fresno CA</t>
+        </is>
+      </c>
+      <c r="I153" t="n">
+        <v>100</v>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>furnace repair Fresno CA</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Columbus Plumbing &amp; Drain</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>columbusplumbingdrain.com</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>https://www.columbusplumbingdrain.com/</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr"/>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>inbound@columbusplumbingdrain.com</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>(614) 879-3783</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Columbus OH</t>
+        </is>
+      </c>
+      <c r="I154" t="n">
+        <v>90</v>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>plumbing company Columbus OH</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 13:25 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L154"/>
+  <dimension ref="A1:L156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9289,7 +9289,6 @@
           <t>https://totallycomfortable.com/furnace-repair/</t>
         </is>
       </c>
-      <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr">
         <is>
           <t>heatingcoolingca@gmail.com</t>
@@ -9345,7 +9344,6 @@
           <t>https://www.columbusplumbingdrain.com/</t>
         </is>
       </c>
-      <c r="E154" t="inlineStr"/>
       <c r="F154" t="inlineStr">
         <is>
           <t>inbound@columbusplumbingdrain.com</t>
@@ -9375,6 +9373,122 @@
         </is>
       </c>
       <c r="L154" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Ace Cooling, Heating, Plumbing and Electrical</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>acehomeaz.com</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>https://acehomeaz.com/areas-served/phoenix-az/hvac-services/furnaces/</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr"/>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>info@acehomeaz.com</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>(928) 851-8704</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="I155" t="n">
+        <v>100</v>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>furnace repair Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Plumber in Winston-Salem, NC | Emergency Plumbing, Drain Cleaning &amp; Water Heater</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>ncplumberdirectory.com</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>https://ncplumberdirectory.com/winston-salem-nc/</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Homeowner Checklist</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>hello@ncplumberdirectory.com</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>866-692-4322</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="I156" t="n">
+        <v>90</v>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>emergency plumber Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 13:27 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L156"/>
+  <dimension ref="A1:L159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9399,7 +9399,6 @@
           <t>https://acehomeaz.com/areas-served/phoenix-az/hvac-services/furnaces/</t>
         </is>
       </c>
-      <c r="E155" t="inlineStr"/>
       <c r="F155" t="inlineStr">
         <is>
           <t>info@acehomeaz.com</t>
@@ -9489,6 +9488,186 @@
         </is>
       </c>
       <c r="L156" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Gonzalez Roofing &amp; Architectural Sheet Metal | Huntsville AL</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>huntsvilleroofingandmetals.com</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>https://www.huntsvilleroofingandmetals.com/</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Sheet Metal</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>sergio@gonzalezroofing.net</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>(256) 513-1990</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>Huntsville AL</t>
+        </is>
+      </c>
+      <c r="I157" t="n">
+        <v>100</v>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Huntsville AL</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Rocket Roofing</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>roofwithrocket.com</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>https://roofwithrocket.com/locations/huntsville-al/</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Repair Repair</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>contact@roofwithrocket.com</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>256-801-7881</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>Huntsville AL</t>
+        </is>
+      </c>
+      <c r="I158" t="n">
+        <v>100</v>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Huntsville AL</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Metal Roofing in Huntsville, AL | 1 Stop Roofing</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>1stoproofingandexteriors.com</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>https://www.1stoproofingandexteriors.com/metal-roofing-huntsville-al.html</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>North Alabama</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>1stopqdc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>256-424-2744</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>Huntsville AL</t>
+        </is>
+      </c>
+      <c r="I159" t="n">
+        <v>90</v>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Huntsville AL</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 13:28 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L159"/>
+  <dimension ref="A1:L161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9673,6 +9673,122 @@
         </is>
       </c>
     </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Best HVAC Company in Salinas, CA - Trusted Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>hvacsalinas.com</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>https://www.hvacsalinas.com/</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Homeowner We</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>info@hvacsalinas.com</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>(831) 329-0462</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>Salinas CA</t>
+        </is>
+      </c>
+      <c r="I160" t="n">
+        <v>100</v>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>HVAC contractor Salinas CA</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Velocity Roofing</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>velocityroofing.com</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>https://velocityroofing.com/service-areas/velocityroofing-roswell-ga/</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Founders Velocity</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>info@velocityroofing.com</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr"/>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>Roswell GA</t>
+        </is>
+      </c>
+      <c r="I161" t="n">
+        <v>76</v>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>residential roofing company Roswell GA</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 13:30 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L161"/>
+  <dimension ref="A1:L163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9764,7 +9764,6 @@
           <t>info@velocityroofing.com</t>
         </is>
       </c>
-      <c r="G161" t="inlineStr"/>
       <c r="H161" t="inlineStr">
         <is>
           <t>Roswell GA</t>
@@ -9784,6 +9783,118 @@
         </is>
       </c>
       <c r="L161" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Plumbing Richardson TX Pro</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>plumbingrichardson-tx.com</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>https://plumbingrichardson-tx.com/sewer-repair.html</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr"/>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>service@plumbingrichardson-tx.com</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>469-213-6752</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>Richardson TX</t>
+        </is>
+      </c>
+      <c r="I162" t="n">
+        <v>100</v>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>sewer repair Richardson TX</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Sewell Plumbing Redesign</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>sewellplumbingtx.com</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>https://sewellplumbingtx.com/richardson-tx-sewer-repairs/</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr"/>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>sewellplumbingtx@gmail.com</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>(214) 606-7648</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>Richardson TX</t>
+        </is>
+      </c>
+      <c r="I163" t="n">
+        <v>90</v>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>sewer repair Richardson TX</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 13:33 UTC (cycle 14)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L163"/>
+  <dimension ref="A1:L166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9809,7 +9809,6 @@
           <t>https://plumbingrichardson-tx.com/sewer-repair.html</t>
         </is>
       </c>
-      <c r="E162" t="inlineStr"/>
       <c r="F162" t="inlineStr">
         <is>
           <t>service@plumbingrichardson-tx.com</t>
@@ -9865,7 +9864,6 @@
           <t>https://sewellplumbingtx.com/richardson-tx-sewer-repairs/</t>
         </is>
       </c>
-      <c r="E163" t="inlineStr"/>
       <c r="F163" t="inlineStr">
         <is>
           <t>sewellplumbingtx@gmail.com</t>
@@ -9895,6 +9893,186 @@
         </is>
       </c>
       <c r="L163" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Keown Builders</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>keownbuilders.com</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>https://keownbuilders.com/residential-roofing-services-frisco-tx/</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>North Texas</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>info@keownbuilders.com</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>(972)748-7661</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Frisco TX</t>
+        </is>
+      </c>
+      <c r="I164" t="n">
+        <v>100</v>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>residential roofing company Frisco TX</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Roofing Services in Frisco, TX | General Roofing</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>generalroofingtexas.com</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>https://generalroofingtexas.com/frisco</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>General Roofing</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>generalroofings@gmail.com</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>469-927-7945</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Frisco TX</t>
+        </is>
+      </c>
+      <c r="I165" t="n">
+        <v>90</v>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>residential roofing company Frisco TX</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Affordable Drain Cleaning in Fontana, CA 92335</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>plumberviews.com</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>https://plumberviews.com/California/fontana-ca-92335/services/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Experience Plumber</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>contact@plumberviews.com</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>(833) 659-1313</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>Fontana CA</t>
+        </is>
+      </c>
+      <c r="I166" t="n">
+        <v>90</v>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>drain cleaning service Fontana CA</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 13:36 UTC (cycle 16)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L166"/>
+  <dimension ref="A1:L168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10078,6 +10078,126 @@
         </is>
       </c>
     </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Cowboys Air Conditioning &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>cowboysac.com</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>https://cowboysac.com/</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Authorized Trane</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>info@cowboysac.com</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>(210) 495-7771</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>San Antonio TX</t>
+        </is>
+      </c>
+      <c r="I167" t="n">
+        <v>100</v>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>HVAC contractor San Antonio TX</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Texas Air HVAC Mechanical LLC</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>texasairhvac.com</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>https://texasairhvac.com/</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>New Braunfels</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>texasairhvacmech@gmail.com</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>(210) 580-4468</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>San Antonio TX</t>
+        </is>
+      </c>
+      <c r="I168" t="n">
+        <v>94</v>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>HVAC contractor San Antonio TX</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 13:42 UTC (cycle 20)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L168"/>
+  <dimension ref="A1:L170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10198,6 +10198,126 @@
         </is>
       </c>
     </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>RiverCity Plumbing</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>rivercityplumbingjax.com</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>https://rivercityplumbingjax.com/services/sewer-line-repair/</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Nadav Far</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>office@rivercityplumbingjax.com</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>(904) 760-7837</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="I169" t="n">
+        <v>90</v>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>sewer repair Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Trenchless Drilling</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>trenchlessdrilling.us</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>https://trenchlessdrilling.us/sewer-line-replacement-jacksonville/</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Free Estimate</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>drilling@trenchlessdrilling.us</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>(305) 600-1734</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="I170" t="n">
+        <v>84</v>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>sewer repair Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 13:43 UTC (cycle 21)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L170"/>
+  <dimension ref="A1:L171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10318,6 +10318,62 @@
         </is>
       </c>
     </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Quality HVAC by Fivid</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>qualityhvac365.com</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>https://qualityhvac365.com/joliet-il-hvac-contractor/</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr"/>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>info@qualityhvac365.com</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>(855) 789-4822</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Joliet IL</t>
+        </is>
+      </c>
+      <c r="I171" t="n">
+        <v>86</v>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>HVAC contractor Joliet IL</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 13:48 UTC (cycle 24)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L171"/>
+  <dimension ref="A1:L172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10339,7 +10339,6 @@
           <t>https://qualityhvac365.com/joliet-il-hvac-contractor/</t>
         </is>
       </c>
-      <c r="E171" t="inlineStr"/>
       <c r="F171" t="inlineStr">
         <is>
           <t>info@qualityhvac365.com</t>
@@ -10369,6 +10368,62 @@
         </is>
       </c>
       <c r="L171" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Clarksburg Plumbing</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>clarksburgplumbing.com</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>https://clarksburgplumbing.com/service-area/germantown/</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr"/>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>office@clarksburgplumbing.com</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>(301) 972 2223</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Germantown MD</t>
+        </is>
+      </c>
+      <c r="I172" t="n">
+        <v>90</v>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>plumber Germantown MD</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 13:52 UTC (cycle 27)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L172"/>
+  <dimension ref="A1:L173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10394,7 +10394,6 @@
           <t>https://clarksburgplumbing.com/service-area/germantown/</t>
         </is>
       </c>
-      <c r="E172" t="inlineStr"/>
       <c r="F172" t="inlineStr">
         <is>
           <t>office@clarksburgplumbing.com</t>
@@ -10424,6 +10423,62 @@
         </is>
       </c>
       <c r="L172" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Metal Roof Services in Bismarck - Roof Rescue ND</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>roofrescuend.com</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>https://roofrescuend.com/services/metal-roof-services</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr"/>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>roofrescuend@gmail.com</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>(701) 870-2956</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Bismarck ND</t>
+        </is>
+      </c>
+      <c r="I173" t="n">
+        <v>86</v>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Bismarck ND</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 13:56 UTC (cycle 30)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L173"/>
+  <dimension ref="A1:L174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10449,7 +10449,6 @@
           <t>https://roofrescuend.com/services/metal-roof-services</t>
         </is>
       </c>
-      <c r="E173" t="inlineStr"/>
       <c r="F173" t="inlineStr">
         <is>
           <t>roofrescuend@gmail.com</t>
@@ -10479,6 +10478,62 @@
         </is>
       </c>
       <c r="L173" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>AccuAir Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>accuairheat.com</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>https://accuairheat.com/city/bend-or/</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr"/>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>accuair@accuairheat.com</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>541-504-8400</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Bend OR</t>
+        </is>
+      </c>
+      <c r="I174" t="n">
+        <v>90</v>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>heating and cooling company Bend OR</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 14:11 UTC (cycle 40)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L174"/>
+  <dimension ref="A1:L175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10504,7 +10504,6 @@
           <t>https://accuairheat.com/city/bend-or/</t>
         </is>
       </c>
-      <c r="E174" t="inlineStr"/>
       <c r="F174" t="inlineStr">
         <is>
           <t>accuair@accuairheat.com</t>
@@ -10534,6 +10533,66 @@
         </is>
       </c>
       <c r="L174" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Quality Works Inc.</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>qualityworksinc.com</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>https://qualityworksinc.com/metal-roofing-boise-id/</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Most Homeowners</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>user@website.com</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>208-608-0943</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>Boise ID</t>
+        </is>
+      </c>
+      <c r="I175" t="n">
+        <v>80</v>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Boise ID</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 14:12 UTC (cycle 41)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L175"/>
+  <dimension ref="A1:L177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10598,6 +10598,122 @@
         </is>
       </c>
     </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>SWAN Plumbing, Heating &amp; Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>swanheating.com</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>https://swanheating.com/aurora-co/</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr"/>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>office@swanheating.com</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>(720) 303-2537</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>Aurora CO</t>
+        </is>
+      </c>
+      <c r="I176" t="n">
+        <v>100</v>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>heating and cooling company Aurora CO</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Goral Construction LLC</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>roofing-goral.com</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>https://roofing-goral.com/service-areas/troy/</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Owner Maciej</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>goralconstruction.llc@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>(248) 804-6933</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Troy MI</t>
+        </is>
+      </c>
+      <c r="I177" t="n">
+        <v>90</v>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>roofing contractor Troy MI</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 14:15 UTC (cycle 43)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L177"/>
+  <dimension ref="A1:L179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10619,7 +10619,6 @@
           <t>https://swanheating.com/aurora-co/</t>
         </is>
       </c>
-      <c r="E176" t="inlineStr"/>
       <c r="F176" t="inlineStr">
         <is>
           <t>office@swanheating.com</t>
@@ -10709,6 +10708,126 @@
         </is>
       </c>
       <c r="L177" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Best HVAC Company in Dearborn, MI - Trusted Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>hvaccontractordearborn.com</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>https://www.hvaccontractordearborn.com/</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Wyoming Ave</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>info@hvaccontractordearborn.com</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>(313) 889-7410</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>Dearborn MI</t>
+        </is>
+      </c>
+      <c r="I178" t="n">
+        <v>100</v>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>heating and cooling company Dearborn MI</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Roofing Services Clarksville TN | JJ Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>jjroofingandrenovations.com</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>https://jjroofingandrenovations.com/</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>jefreyrivera10@gmail.com</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>(901) 643-0903</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>Clarksville TN</t>
+        </is>
+      </c>
+      <c r="I179" t="n">
+        <v>90</v>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>residential roofing company Clarksville TN</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 14:26 UTC (cycle 50)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L179"/>
+  <dimension ref="A1:L180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10833,6 +10833,66 @@
         </is>
       </c>
     </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Top Edge Roofing</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>topedgeroofing.com</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>https://topedgeroofing.com/</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Free Roof</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>info@topedgeroofing.com</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>(406)570-0832</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>Bozeman MT</t>
+        </is>
+      </c>
+      <c r="I180" t="n">
+        <v>90</v>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>roofing contractor Bozeman MT</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 14:30 UTC (cycle 53)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L180"/>
+  <dimension ref="A1:L182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10893,6 +10893,126 @@
         </is>
       </c>
     </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Canyon State Roofing &amp; Consulting - YOUR Arizona Roofing Company</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>canyonstateroofs.com</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>https://canyonstateroofs.com/services/where-we-work/gilbert-roofers/</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Bruce Ave</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>info@canyonstateroofs.com</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>602-400-1635</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="I181" t="n">
+        <v>100</v>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>roof repair company Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Montana Pro Contractors</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>mpc-roofing.com</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>https://www.mpc-roofing.com/greatfalls</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Why Great</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>sales@mpc-roofing.com</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>406-880-2511</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>Great Falls MT</t>
+        </is>
+      </c>
+      <c r="I182" t="n">
+        <v>90</v>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Great Falls MT</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 14:33 UTC (cycle 55)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L182"/>
+  <dimension ref="A1:L183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11013,6 +11013,66 @@
         </is>
       </c>
     </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Custom Cooling &amp; Contracting</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>customcoolingtx.com</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>https://customcoolingtx.com/mesquite</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Custom Cooling</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>customcoolingtx@gmail.com</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>469-588-7750</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>Mesquite TX</t>
+        </is>
+      </c>
+      <c r="I183" t="n">
+        <v>86</v>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>heating and cooling company Mesquite TX</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 14:42 UTC (cycle 61)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L183"/>
+  <dimension ref="A1:L184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11073,6 +11073,66 @@
         </is>
       </c>
     </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Galloroofingllc.</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>galloroofingllc.com</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>https://galloroofingllc.com/surprise/</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Commercial Sales</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>office@galloroofing.net</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>(602) 533-0013</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>Surprise AZ</t>
+        </is>
+      </c>
+      <c r="I184" t="n">
+        <v>100</v>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>residential roofing company Surprise AZ</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 14:54 UTC (cycle 69)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L184"/>
+  <dimension ref="A1:L185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11133,6 +11133,66 @@
         </is>
       </c>
     </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Tridom Roofing</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>tridomroofing.com</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>https://www.tridomroofing.com/locations/roofing-austin-texas/residential/</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Residential Roofing</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>info@tridomroofing.com</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>(844) 887-4366</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>Austin TX</t>
+        </is>
+      </c>
+      <c r="I185" t="n">
+        <v>100</v>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>residential roofing company Austin TX</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 14:55 UTC (cycle 70)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L185"/>
+  <dimension ref="A1:L186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11193,6 +11193,66 @@
         </is>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>AirHeads HVAC</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>airheadshvac.com</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>https://airheadshvac.com/city/killeen-tx/</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Comfort Club</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>office@airheadshvac.com</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>254-213-5400</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>Killeen TX</t>
+        </is>
+      </c>
+      <c r="I186" t="n">
+        <v>90</v>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>heat pump installation Killeen TX</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 14:58 UTC (cycle 72)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L186"/>
+  <dimension ref="A1:L187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11253,6 +11253,62 @@
         </is>
       </c>
     </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Plumbing Company, Local Plumbers | Archie's Plumbing | Billings &amp; Laurel, MT</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>archiesplumbingbillings.com</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>https://www.archiesplumbingbillings.com/</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr"/>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>api.contracting23@gmail.com</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>(406) 598-8820</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>Billings MT</t>
+        </is>
+      </c>
+      <c r="I187" t="n">
+        <v>88</v>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>plumbing company Billings MT</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 15:04 UTC (cycle 76)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L187"/>
+  <dimension ref="A1:L189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11274,7 +11274,6 @@
           <t>https://www.archiesplumbingbillings.com/</t>
         </is>
       </c>
-      <c r="E187" t="inlineStr"/>
       <c r="F187" t="inlineStr">
         <is>
           <t>api.contracting23@gmail.com</t>
@@ -11304,6 +11303,122 @@
         </is>
       </c>
       <c r="L187" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>JLB Roofing</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>jlbroofingcompany.com</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>https://jlbroofingcompany.com/sandy-ut/</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr"/>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>john@gmail.com</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>(801) 645-1647</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>Sandy UT</t>
+        </is>
+      </c>
+      <c r="I188" t="n">
+        <v>100</v>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>roof repair company Sandy UT</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Revive Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>reviveroofingut.com</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>https://reviveroofingut.com/service-areas/sandy/</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Salt Lake</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>info@reviveroofingut.com</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>(801) 421-6336</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>Sandy UT</t>
+        </is>
+      </c>
+      <c r="I189" t="n">
+        <v>90</v>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>roof repair company Sandy UT</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 15:07 UTC (cycle 78)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L189"/>
+  <dimension ref="A1:L190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11329,7 +11329,6 @@
           <t>https://jlbroofingcompany.com/sandy-ut/</t>
         </is>
       </c>
-      <c r="E188" t="inlineStr"/>
       <c r="F188" t="inlineStr">
         <is>
           <t>john@gmail.com</t>
@@ -11419,6 +11418,66 @@
         </is>
       </c>
       <c r="L189" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Westside Plumbing</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>westsideplumbingca.com</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>https://westsideplumbingca.com/services/water-heater</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Areas Contact</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>info@westsideplumbingca.com</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>(209) 622-5723</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Modesto CA</t>
+        </is>
+      </c>
+      <c r="I190" t="n">
+        <v>90</v>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>water heater repair Modesto CA</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L190" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 15:09 UTC (cycle 79)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L190"/>
+  <dimension ref="A1:L191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11483,6 +11483,66 @@
         </is>
       </c>
     </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Shelley Construction Roofing</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>shelley-construction.com</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>https://shelley-construction.com/service-area/orem</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Free Estimate</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>info@shelley-construction.com</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>(385) 347-0568</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>Orem UT</t>
+        </is>
+      </c>
+      <c r="I191" t="n">
+        <v>90</v>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>roof replacement Orem UT</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 15:10 UTC (cycle 80)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L191"/>
+  <dimension ref="A1:L192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11543,6 +11543,62 @@
         </is>
       </c>
     </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Drain Cleaning in Sandy Springs, GA - Superior Plumbing</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>draincleaningsandyspringsga.com</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>https://www.draincleaningsandyspringsga.com/</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr"/>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>customerservice@superiorplumbing.com</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>770-422-7586</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>Sandy Springs GA</t>
+        </is>
+      </c>
+      <c r="I192" t="n">
+        <v>100</v>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>drain cleaning service Sandy Springs GA</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 15:19 UTC (cycle 86)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L192"/>
+  <dimension ref="A1:L193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11564,7 +11564,6 @@
           <t>https://www.draincleaningsandyspringsga.com/</t>
         </is>
       </c>
-      <c r="E192" t="inlineStr"/>
       <c r="F192" t="inlineStr">
         <is>
           <t>customerservice@superiorplumbing.com</t>
@@ -11594,6 +11593,66 @@
         </is>
       </c>
       <c r="L192" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Expert Roofing of Westchester</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>expertroofingwestchester.com</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>https://expertroofingwestchester.com/</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Hudson Valley</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>info@expertroofingwestchester.com</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>914-446-3072</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Yonkers NY</t>
+        </is>
+      </c>
+      <c r="I193" t="n">
+        <v>100</v>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>roof repair company Yonkers NY</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 15:22 UTC (cycle 88)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L193"/>
+  <dimension ref="A1:L194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11658,6 +11658,66 @@
         </is>
       </c>
     </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Turbo Plumbing &amp; Rooter</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>turboplumbingandrooter.com</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>https://turboplumbingandrooter.com/areas-served/santa-clarita/sewer-lines/</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Review Rapid</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>info@turboplumbingandrooter.com</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>(213) 423-4167</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>Santa Clarita CA</t>
+        </is>
+      </c>
+      <c r="I194" t="n">
+        <v>100</v>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>sewer repair Santa Clarita CA</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 15:25 UTC (cycle 90)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L194"/>
+  <dimension ref="A1:L196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11718,6 +11718,122 @@
         </is>
       </c>
     </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>bestiniownrochesterplumbing.com</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>bestiniownrochesterplumbing.com</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>https://bestiniownrochesterplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Hours Plumbing</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>aman@a8c.in</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>(585) 438-8500</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>Rochester NY</t>
+        </is>
+      </c>
+      <c r="I195" t="n">
+        <v>100</v>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>emergency plumber Rochester NY</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Leone Plumbing and Heating</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>leoneservice.com</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>https://www.leoneservice.com/rochester-ny/emergency-plumbing-services/</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr"/>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>contact@leoneservice.com</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>(585) 458-5800</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>Rochester NY</t>
+        </is>
+      </c>
+      <c r="I196" t="n">
+        <v>90</v>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>emergency plumber Rochester NY</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 15:29 UTC (cycle 93)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L196"/>
+  <dimension ref="A1:L198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11799,7 +11799,6 @@
           <t>https://www.leoneservice.com/rochester-ny/emergency-plumbing-services/</t>
         </is>
       </c>
-      <c r="E196" t="inlineStr"/>
       <c r="F196" t="inlineStr">
         <is>
           <t>contact@leoneservice.com</t>
@@ -11829,6 +11828,126 @@
         </is>
       </c>
       <c r="L196" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Roofing in Columbia  MD - Robust Roof</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>robustroof.com</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>https://www.robustroof.com/roofing-columbia-md</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>John Clark</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>jclark@robustroof.com</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>555-555-5555</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>Columbia MD</t>
+        </is>
+      </c>
+      <c r="I197" t="n">
+        <v>100</v>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>roofer Columbia MD</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Plumbing Anaheim CA | Oc x La Plumbing</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>ocxlaplumbing.com</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>https://www.ocxlaplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>La Plumbing</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>ocxlaplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>(714) 366-7618</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Anaheim CA</t>
+        </is>
+      </c>
+      <c r="I198" t="n">
+        <v>90</v>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>plumbing company Anaheim CA</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 15:35 UTC (cycle 97)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L198"/>
+  <dimension ref="A1:L200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11953,6 +11953,122 @@
         </is>
       </c>
     </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Bean'z Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>beanzheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>https://beanzheatingandcooling.com/furnace-repair-service-chicago/</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Company Chicago</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>beanzheatingandcooling@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>312-593-6334</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>Chicago IL</t>
+        </is>
+      </c>
+      <c r="I199" t="n">
+        <v>90</v>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>furnace repair Chicago IL</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Sunset Heating and Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>sunsetheatingandairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>https://sunsetheatingandairconditioning.com/furnace-repair-chicago-il</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr"/>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>micah@micahrich.com</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>708-397-6644</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>Chicago IL</t>
+        </is>
+      </c>
+      <c r="I200" t="n">
+        <v>80</v>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>furnace repair Chicago IL</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 15:56 UTC (cycle 111)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L200"/>
+  <dimension ref="A1:L202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -12034,7 +12034,6 @@
           <t>https://sunsetheatingandairconditioning.com/furnace-repair-chicago-il</t>
         </is>
       </c>
-      <c r="E200" t="inlineStr"/>
       <c r="F200" t="inlineStr">
         <is>
           <t>micah@micahrich.com</t>
@@ -12064,6 +12063,122 @@
         </is>
       </c>
       <c r="L200" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>carterroofingremodeling.pro</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>carterroofingremodeling.pro</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>https://carterroofingremodeling.pro/roof-replacement-pasadena-tx/</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Story Professional</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>khatodiasahil3@gmail.com</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>(832) 536-6528</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>Pasadena TX</t>
+        </is>
+      </c>
+      <c r="I201" t="n">
+        <v>90</v>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>roof replacement Pasadena TX</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>AO1 Roofing Company</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>ao1roofingandconstruction.com</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>https://ao1roofingandconstruction.com/roof-replacement-in-pasadena-texas/</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Team Member</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>info@ao1roofing.com</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr"/>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>Pasadena TX</t>
+        </is>
+      </c>
+      <c r="I202" t="n">
+        <v>76</v>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>roof replacement Pasadena TX</t>
+        </is>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 16:02 UTC (cycle 115)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L202"/>
+  <dimension ref="A1:L204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -12159,7 +12159,6 @@
           <t>info@ao1roofing.com</t>
         </is>
       </c>
-      <c r="G202" t="inlineStr"/>
       <c r="H202" t="inlineStr">
         <is>
           <t>Pasadena TX</t>
@@ -12179,6 +12178,126 @@
         </is>
       </c>
       <c r="L202" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Acme Roofing</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>estimate.acmeroofingwa.com</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>https://estimate.acmeroofingwa.com/roof-replacement-federal-way-wa/</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Expert Local</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>general@acmeroofingwa.com</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>(253) 564-2292</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>Federal Way WA</t>
+        </is>
+      </c>
+      <c r="I203" t="n">
+        <v>100</v>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>roof replacement Federal Way WA</t>
+        </is>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Roofing &amp; Siding Contractors | Columbia, MO | Signature Exteriors</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>signatureext.com</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>https://signatureext.com/columbia-mo</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Boone County</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>projects@signatureext.com</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>509.295.8066</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>Columbia MO</t>
+        </is>
+      </c>
+      <c r="I204" t="n">
+        <v>90</v>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>roof replacement Columbia MO</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L204" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 16:03 UTC (cycle 116)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L204"/>
+  <dimension ref="A1:L205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -12303,6 +12303,66 @@
         </is>
       </c>
     </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>All-in-One Drain Solutions: Choose from Expert Service Companies</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>draincleaningservicecompanies.com</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>https://draincleaningservicecompanies.com/drain-cleaning-jacksonville-fl/</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Clogged Drain</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>contact@draincleaningservicecompanies.com</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>(888) 994-0172</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="I205" t="n">
+        <v>90</v>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>drain cleaning service Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 16:22 UTC (cycle 129)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L205"/>
+  <dimension ref="A1:L206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -12363,6 +12363,66 @@
         </is>
       </c>
     </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Everguard Roofing</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>everguardroofing.com</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>https://everguardroofing.com/</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Peggy Norton</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>thebestroof@everguardroofing.com</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>(505) 821-9543</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="I206" t="n">
+        <v>90</v>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>roof repair company Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 16:37 UTC (cycle 139)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L206"/>
+  <dimension ref="A1:L208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -12423,6 +12423,118 @@
         </is>
       </c>
     </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Bertucci Bros NOLA</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>bertuccibrothersplumbing.com</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>https://www.bertuccibrothersplumbing.com/plumbers-metairie</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr"/>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>figgy830@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>(504) 559 7473</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>Metairie LA</t>
+        </is>
+      </c>
+      <c r="I207" t="n">
+        <v>100</v>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>plumber Metairie LA</t>
+        </is>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Residential Roofing Company | Toledo, OH | RoofOhio</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>roofohio.com</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>https://www.roofohio.com/contact/residential-roofing-company-service-area/toledo-oh</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr"/>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>office@roofohio.com</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>(419) 865-1799</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>Toledo OH</t>
+        </is>
+      </c>
+      <c r="I208" t="n">
+        <v>90</v>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>residential roofing company Toledo OH</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 16:40 UTC (cycle 141)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L208"/>
+  <dimension ref="A1:L210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -12444,7 +12444,6 @@
           <t>https://www.bertuccibrothersplumbing.com/plumbers-metairie</t>
         </is>
       </c>
-      <c r="E207" t="inlineStr"/>
       <c r="F207" t="inlineStr">
         <is>
           <t>figgy830@yahoo.com</t>
@@ -12500,7 +12499,6 @@
           <t>https://www.roofohio.com/contact/residential-roofing-company-service-area/toledo-oh</t>
         </is>
       </c>
-      <c r="E208" t="inlineStr"/>
       <c r="F208" t="inlineStr">
         <is>
           <t>office@roofohio.com</t>
@@ -12530,6 +12528,122 @@
         </is>
       </c>
       <c r="L208" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Advanced Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>advancedacnow.com</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>https://advancedacnow.com/services/ac-repair-orlando/</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr"/>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>info@advancedacnow.com</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>407-604-0279</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>Orlando FL</t>
+        </is>
+      </c>
+      <c r="I209" t="n">
+        <v>100</v>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>air conditioning repair Orlando FL</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Fort Wayne Roofing</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>fortwayneinroofing.com</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>https://fortwayneinroofing.com/</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Schedule Free</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>info@fortwayneinroofing.com</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>(260) 201-2585</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="I210" t="n">
+        <v>96</v>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>roofing contractor Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 16:41 UTC (cycle 142)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L210"/>
+  <dimension ref="A1:L211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -12554,7 +12554,6 @@
           <t>https://advancedacnow.com/services/ac-repair-orlando/</t>
         </is>
       </c>
-      <c r="E209" t="inlineStr"/>
       <c r="F209" t="inlineStr">
         <is>
           <t>info@advancedacnow.com</t>
@@ -12644,6 +12643,62 @@
         </is>
       </c>
       <c r="L210" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Trusted HVAC Experts | Independence, MO</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>mcintosh-hc.com</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>https://www.mcintosh-hc.com/</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr"/>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>info@mcintosh-hc.com</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>816-373-9500</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>Independence MO</t>
+        </is>
+      </c>
+      <c r="I211" t="n">
+        <v>88</v>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>heating and cooling company Independence MO</t>
+        </is>
+      </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L211" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 16:47 UTC (cycle 146)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L211"/>
+  <dimension ref="A1:L212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -12669,7 +12669,6 @@
           <t>https://www.mcintosh-hc.com/</t>
         </is>
       </c>
-      <c r="E211" t="inlineStr"/>
       <c r="F211" t="inlineStr">
         <is>
           <t>info@mcintosh-hc.com</t>
@@ -12699,6 +12698,66 @@
         </is>
       </c>
       <c r="L211" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Anna's Air, Heat &amp; Plumbing</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>annasairandheat.com</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>https://www.annasairandheat.com/service-areas/palm-bay-fl</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Indoor Air</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>annasairheatplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>321-307-2820</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="I212" t="n">
+        <v>90</v>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>heating and cooling company Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L212" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 16:50 UTC (cycle 148)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L212"/>
+  <dimension ref="A1:L213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -12763,6 +12763,66 @@
         </is>
       </c>
     </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Heating &amp; AC Service &amp; Repair</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>totalcomfortlansing.com</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>https://www.totalcomfortlansing.com/</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Chris Swope</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>info@totalcomfortlansing.com</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>(517) 484-2122</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>Lansing MI</t>
+        </is>
+      </c>
+      <c r="I213" t="n">
+        <v>78</v>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>heating and cooling company Lansing MI</t>
+        </is>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 16:56 UTC (cycle 152)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L213"/>
+  <dimension ref="A1:L214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -12823,6 +12823,62 @@
         </is>
       </c>
     </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Rogue Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>rogueheatandair.com</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>https://rogueheatandair.com/</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Schedule Quick</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>rogueheatingandair@gmail.com</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr"/>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>Medford OR</t>
+        </is>
+      </c>
+      <c r="I214" t="n">
+        <v>76</v>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>furnace repair Medford OR</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 16:59 UTC (cycle 154)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L214"/>
+  <dimension ref="A1:L215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -12854,7 +12854,6 @@
           <t>rogueheatingandair@gmail.com</t>
         </is>
       </c>
-      <c r="G214" t="inlineStr"/>
       <c r="H214" t="inlineStr">
         <is>
           <t>Medford OR</t>
@@ -12874,6 +12873,66 @@
         </is>
       </c>
       <c r="L214" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Site for migration</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>modernairofkaty.com</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>https://modernairofkaty.com/katy-ac-repair/</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Katy Homeowners</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>charles@modernairofkaty.com</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>713-620-8900</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>Katy TX</t>
+        </is>
+      </c>
+      <c r="I215" t="n">
+        <v>100</v>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>air conditioning repair Katy TX</t>
+        </is>
+      </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L215" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 17:08 UTC (cycle 160)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L215"/>
+  <dimension ref="A1:L216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -12938,6 +12938,66 @@
         </is>
       </c>
     </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Roof Repair Company</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>roof.day</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>https://www.roof.day/service-areas/conroe</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Repair Company</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>office@roof.day</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>713-489-4265</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>Conroe TX</t>
+        </is>
+      </c>
+      <c r="I216" t="n">
+        <v>90</v>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>roof repair company Conroe TX</t>
+        </is>
+      </c>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 17:21 UTC (cycle 169)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L216"/>
+  <dimension ref="A1:L217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -12998,6 +12998,62 @@
         </is>
       </c>
     </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Heating &amp; Air Services Stockton | Greener Solutions</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>gshomeservices.com</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>https://www.gshomeservices.com/furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr"/>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>service@gshomeservices.com</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>(209) 232-8595</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>Stockton CA</t>
+        </is>
+      </c>
+      <c r="I217" t="n">
+        <v>100</v>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>furnace repair Stockton CA</t>
+        </is>
+      </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 17:22 UTC (cycle 170)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L217"/>
+  <dimension ref="A1:L219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -13019,7 +13019,6 @@
           <t>https://www.gshomeservices.com/furnace-repair/</t>
         </is>
       </c>
-      <c r="E217" t="inlineStr"/>
       <c r="F217" t="inlineStr">
         <is>
           <t>service@gshomeservices.com</t>
@@ -13049,6 +13048,126 @@
         </is>
       </c>
       <c r="L217" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Best HVAC Company in Chula Vista, CA - Trusted Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>chulavistahvacpro.com</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>https://chulavistahvacpro.com/</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Chula Vista</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>info@chulavistahvacpro.com</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>(619) 975-3557</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>Chula Vista CA</t>
+        </is>
+      </c>
+      <c r="I218" t="n">
+        <v>100</v>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>heating and cooling company Chula Vista CA</t>
+        </is>
+      </c>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Trusted AC Service in Warwick, RI</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>greenwoodplumbingandheating.com</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>https://greenwoodplumbingandheating.com/trusted-ac-service-in-warwick-ri-reliable-ac-repair/</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Repair Trusted</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>mrrooterofri@gmail.com</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>401.738.9245</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>Warwick RI</t>
+        </is>
+      </c>
+      <c r="I219" t="n">
+        <v>90</v>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>air conditioning repair Warwick RI</t>
+        </is>
+      </c>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L219" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 17:28 UTC (cycle 174)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L219"/>
+  <dimension ref="A1:L221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -13173,6 +13173,126 @@
         </is>
       </c>
     </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>EZ Plumbing &amp; Repair</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>ezplumbingandrepair.com</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>https://www.ezplumbingandrepair.com/tn-water-heater</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>What Our</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>info@ezplumbingandrepair.com</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>423-275-5500</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>Chattanooga TN</t>
+        </is>
+      </c>
+      <c r="I220" t="n">
+        <v>90</v>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>water heater repair Chattanooga TN</t>
+        </is>
+      </c>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Water Heater Repair in Chattanooga, TN | Free Diagnosis | Perfect Pipe</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>perfectpipeplumbing.com</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>https://perfectpipeplumbing.com/water-heater-repair/tn/chattanooga/</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Get Free</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>service@perfectpipeplumbing.com</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>(423) 325-4137</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>Chattanooga TN</t>
+        </is>
+      </c>
+      <c r="I221" t="n">
+        <v>90</v>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>water heater repair Chattanooga TN</t>
+        </is>
+      </c>
+      <c r="K221" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 17:33 UTC (cycle 177)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L221"/>
+  <dimension ref="A1:L222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -13293,6 +13293,62 @@
         </is>
       </c>
     </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>JJM Roofing &amp; Seamless Gutters</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>jjmhomeremodel.com</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>https://www.jjmhomeremodel.com/metal-roofs/</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr"/>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>jjmroofing@aol.com</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>(585)245-1972</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>Rochester NY</t>
+        </is>
+      </c>
+      <c r="I222" t="n">
+        <v>76</v>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Rochester NY</t>
+        </is>
+      </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 17:34 UTC (cycle 178)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L222"/>
+  <dimension ref="A1:L223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -13314,7 +13314,6 @@
           <t>https://www.jjmhomeremodel.com/metal-roofs/</t>
         </is>
       </c>
-      <c r="E222" t="inlineStr"/>
       <c r="F222" t="inlineStr">
         <is>
           <t>jjmroofing@aol.com</t>
@@ -13344,6 +13343,66 @@
         </is>
       </c>
       <c r="L222" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Jones Heat &amp; Air</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>jonesheatair.com</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>https://jonesheatair.com/service-areas/modesto-ca.html</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Jones Heat</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>jonescomfortzone@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>(209) 632-5675</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>Modesto CA</t>
+        </is>
+      </c>
+      <c r="I223" t="n">
+        <v>90</v>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>heating and cooling company Modesto CA</t>
+        </is>
+      </c>
+      <c r="K223" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L223" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 17:36 UTC (cycle 179)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L223"/>
+  <dimension ref="A1:L224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -13408,6 +13408,66 @@
         </is>
       </c>
     </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>masheatingcooling.com</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>masheatingcooling.com</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>https://masheatingcooling.com/</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>angel21469@gmail.com</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>(214) 530-6579</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>Irving TX</t>
+        </is>
+      </c>
+      <c r="I224" t="n">
+        <v>90</v>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>HVAC contractor Irving TX</t>
+        </is>
+      </c>
+      <c r="K224" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 17:39 UTC (cycle 181)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L224"/>
+  <dimension ref="A1:L225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -13468,6 +13468,66 @@
         </is>
       </c>
     </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>HVAC Service Plano - Ensure Year-Round Comfort with Expert HVAC Services!</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>elementmechanicalac.com</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>https://www.elementmechanicalac.com/service-area/plano/</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Read More</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>ryan@elementmechanicalac.com</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>(972) 771-7522</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>Plano TX</t>
+        </is>
+      </c>
+      <c r="I225" t="n">
+        <v>90</v>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>AC installation Plano TX</t>
+        </is>
+      </c>
+      <c r="K225" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 17:50 UTC (cycle 189)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L225"/>
+  <dimension ref="A1:L226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -13528,6 +13528,66 @@
         </is>
       </c>
     </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Anaheim Roofing Pros</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>anaheimroofingpros.com</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>https://anaheimroofingpros.com/roof-repair-in-anaheim/</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>Anaheim Roofing</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>info@anaheimroofingpros.com</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>(657) 514-5060</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>Anaheim CA</t>
+        </is>
+      </c>
+      <c r="I226" t="n">
+        <v>100</v>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>roof repair company Anaheim CA</t>
+        </is>
+      </c>
+      <c r="K226" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 17:58 UTC (cycle 194)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L226"/>
+  <dimension ref="A1:L228"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -13588,6 +13588,126 @@
         </is>
       </c>
     </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Brownlee Plumbing LLC</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>brownlee.plumbing</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>https://brownlee.plumbing/</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Honest Pricing</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>customersupport@brownleeplumbing.com</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>(703) 477-9016</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>Alexandria VA</t>
+        </is>
+      </c>
+      <c r="I227" t="n">
+        <v>100</v>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>plumbing company Alexandria VA</t>
+        </is>
+      </c>
+      <c r="K227" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>AC Installation in College Station, TX</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>centralairandrefrigeration.com</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>https://www.centralairandrefrigeration.com/feeds/service/ac-installation-college-station-tx</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>Maintenance Contract</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>centralaaservice@gmail.com</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>(979) 324-6791</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>College Station TX</t>
+        </is>
+      </c>
+      <c r="I228" t="n">
+        <v>100</v>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>AC installation College Station TX</t>
+        </is>
+      </c>
+      <c r="K228" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 18:05 UTC (cycle 199)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L228"/>
+  <dimension ref="A1:L229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -13708,6 +13708,62 @@
         </is>
       </c>
     </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Plumbing Services Richardson, TX</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>richardsondraincleaning.com</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>http://richardsondraincleaning.com/</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr"/>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>service@richardsondraincleaning.com</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>972-246-8157</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>Richardson TX</t>
+        </is>
+      </c>
+      <c r="I229" t="n">
+        <v>76</v>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>drain cleaning service Richardson TX</t>
+        </is>
+      </c>
+      <c r="K229" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 18:07 UTC (cycle 200)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L229"/>
+  <dimension ref="A1:L230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -13729,7 +13729,6 @@
           <t>http://richardsondraincleaning.com/</t>
         </is>
       </c>
-      <c r="E229" t="inlineStr"/>
       <c r="F229" t="inlineStr">
         <is>
           <t>service@richardsondraincleaning.com</t>
@@ -13759,6 +13758,66 @@
         </is>
       </c>
       <c r="L229" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>West Valley City Roofing Company | Nelson Roofing Experts</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>nelsonroofingslc.com</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>https://www.nelsonroofingslc.com/west-valley-city</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Salt Lake</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>info@nelsonroofingslc.com</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>(801) 845-3363</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>West Valley City UT</t>
+        </is>
+      </c>
+      <c r="I230" t="n">
+        <v>100</v>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>roofer West Valley City UT</t>
+        </is>
+      </c>
+      <c r="K230" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L230" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 18:12 UTC (cycle 204)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L230"/>
+  <dimension ref="A1:L231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -13823,6 +13823,66 @@
         </is>
       </c>
     </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Roofer in Edison, NJ | Joseph David Roofing</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>jdavidroofing.net</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>https://www.jdavidroofing.net/edison-nj/</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Why Property</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>ldavid@jdavidroofing.net</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>(908) 925-0007</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>Edison NJ</t>
+        </is>
+      </c>
+      <c r="I231" t="n">
+        <v>100</v>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>roofer Edison NJ</t>
+        </is>
+      </c>
+      <c r="K231" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 18:40 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L231"/>
+  <dimension ref="A1:L232"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -13883,6 +13883,66 @@
         </is>
       </c>
     </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>S&amp;R Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>srheatingcooling.com</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>https://www.srheatingcooling.com/air-conditioning-replacement-installation/</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Neighbors Choose</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>srappliance@qwestoffice.net</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>651-429-0001</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>Woodbury MN</t>
+        </is>
+      </c>
+      <c r="I232" t="n">
+        <v>100</v>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>AC installation Woodbury MN</t>
+        </is>
+      </c>
+      <c r="K232" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 18:46 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L232"/>
+  <dimension ref="A1:L234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -13943,6 +13943,122 @@
         </is>
       </c>
     </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Mullen Plumbing, Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>mullenplumbing.com</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>https://mullenplumbing.com/areas-we-serve/charleston-wv/</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>South Charleston</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>tom.orcutt@mullenplumbing.com</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>(304) 744-3221</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>Charleston WV</t>
+        </is>
+      </c>
+      <c r="I233" t="n">
+        <v>100</v>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>heating and cooling company Charleston WV</t>
+        </is>
+      </c>
+      <c r="K233" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Norfolk Air Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>norfolkair-hvac.com</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>https://www.norfolkair-hvac.com/norfolk-air-heating-cooling-services/</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr"/>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>admin@guysmith.net</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>757-963-8365</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>Norfolk VA</t>
+        </is>
+      </c>
+      <c r="I234" t="n">
+        <v>90</v>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>heating and cooling company Norfolk VA</t>
+        </is>
+      </c>
+      <c r="K234" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 18:48 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L234"/>
+  <dimension ref="A1:L237"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -14024,7 +14024,6 @@
           <t>https://www.norfolkair-hvac.com/norfolk-air-heating-cooling-services/</t>
         </is>
       </c>
-      <c r="E234" t="inlineStr"/>
       <c r="F234" t="inlineStr">
         <is>
           <t>admin@guysmith.net</t>
@@ -14054,6 +14053,182 @@
         </is>
       </c>
       <c r="L234" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Stonecreek Roofing</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>stonecreekroofingaz.com</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>https://roofingcompaniesphoenix.com/service-areas/gilbert</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Contractor Gilbert</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>info@stonecreekroofingaz.com</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>(602) 324-3400</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="I235" t="n">
+        <v>90</v>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>roofing contractor Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="K235" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Happy Hippo Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>callhappyhippo.com</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>https://callhappyhippo.com/hvac-services-joliet-il/furnace-repair-joliet-il/</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>All Rights</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>office@callhappyhippo.com</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>(815) 905-8268</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>Joliet IL</t>
+        </is>
+      </c>
+      <c r="I236" t="n">
+        <v>90</v>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>furnace repair Joliet IL</t>
+        </is>
+      </c>
+      <c r="K236" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>North West Premier Roofing</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>bellingham-wa.northwestpremierroofing.com</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>https://bellingham-wa.northwestpremierroofing.com/</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr"/>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>info@northwestpremierroofing.com</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>(360) 803-0369</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>Bellingham WA</t>
+        </is>
+      </c>
+      <c r="I237" t="n">
+        <v>90</v>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>residential roofing company Bellingham WA</t>
+        </is>
+      </c>
+      <c r="K237" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L237" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 18:49 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L237"/>
+  <dimension ref="A1:L240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -14199,7 +14199,6 @@
           <t>https://bellingham-wa.northwestpremierroofing.com/</t>
         </is>
       </c>
-      <c r="E237" t="inlineStr"/>
       <c r="F237" t="inlineStr">
         <is>
           <t>info@northwestpremierroofing.com</t>
@@ -14229,6 +14228,182 @@
         </is>
       </c>
       <c r="L237" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>American Air Cares, Inc.</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>americanaircares.com</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>https://americanaircares.com/</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr"/>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>info@americanaircares.com</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>772-398-0023</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>Port St Lucie FL</t>
+        </is>
+      </c>
+      <c r="I238" t="n">
+        <v>100</v>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>heating and cooling company Port St Lucie FL</t>
+        </is>
+      </c>
+      <c r="K238" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Metro Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>metrohci.com</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>https://metrohci.com/service/ac-installation/</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Are Metro</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>info@metrohci.com</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>(515) 266-3693</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>Des Moines IA</t>
+        </is>
+      </c>
+      <c r="I239" t="n">
+        <v>100</v>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>AC installation Des Moines IA</t>
+        </is>
+      </c>
+      <c r="K239" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>A/C Care Heat &amp; Air</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>accareheatair.com</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>https://accareheatair.com/hvac-port-st-lucie/</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Care Heat</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>office@accare.biz</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>(772) 232-5266</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>Port St Lucie FL</t>
+        </is>
+      </c>
+      <c r="I240" t="n">
+        <v>100</v>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>heating and cooling company Port St Lucie FL</t>
+        </is>
+      </c>
+      <c r="K240" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L240" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 18:55 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L240"/>
+  <dimension ref="A1:L241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -14254,7 +14254,6 @@
           <t>https://americanaircares.com/</t>
         </is>
       </c>
-      <c r="E238" t="inlineStr"/>
       <c r="F238" t="inlineStr">
         <is>
           <t>info@americanaircares.com</t>
@@ -14404,6 +14403,66 @@
         </is>
       </c>
       <c r="L240" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Elite Air Service</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>eliteairserviceca.com</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>https://eliteairserviceca.com/residential-air-conditioning-heating-bakersfield-ca/</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>Owner Tim</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>eliteairservice@hotmail.com</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>(661) 410-8390</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>Bakersfield CA</t>
+        </is>
+      </c>
+      <c r="I241" t="n">
+        <v>90</v>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>heating and cooling company Bakersfield CA</t>
+        </is>
+      </c>
+      <c r="K241" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L241" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 18:58 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L241"/>
+  <dimension ref="A1:L242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -14468,6 +14468,66 @@
         </is>
       </c>
     </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Reno AC Repair and Heating | Reno, NV HVAC Experts</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>renoacrepairandheating.com</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>https://renoacrepairandheating.com/</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>Why Choose</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>info@renoacrepairandheating.com</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>(775) 218-1564</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>Reno NV</t>
+        </is>
+      </c>
+      <c r="I242" t="n">
+        <v>90</v>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>air conditioning repair Reno NV</t>
+        </is>
+      </c>
+      <c r="K242" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 18:59 UTC (cycle 14)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L242"/>
+  <dimension ref="A1:L244"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -14528,6 +14528,126 @@
         </is>
       </c>
     </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Progressive Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>progressiveairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>https://progressiveairconditioning.com/heat-pump/heat-pump-installation-replacement-chula-vista-ca</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>Chula Vista</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>office@arcticairflow.com</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>(858) 529-5050</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>Chula Vista CA</t>
+        </is>
+      </c>
+      <c r="I243" t="n">
+        <v>100</v>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>heat pump installation Chula Vista CA</t>
+        </is>
+      </c>
+      <c r="K243" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>The Roof Doctor</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>louisvilleroofdoctor.com</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>https://louisvilleroofdoctor.com/louisville-roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>Roof Doctor</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>info@louisvilleroofdoctor.com</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>(502) 458-2345</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>Louisville KY</t>
+        </is>
+      </c>
+      <c r="I244" t="n">
+        <v>88</v>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>roof replacement Louisville KY</t>
+        </is>
+      </c>
+      <c r="K244" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 19:02 UTC (cycle 16)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L244"/>
+  <dimension ref="A1:L245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -14648,6 +14648,62 @@
         </is>
       </c>
     </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation in Richardson TX</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>planohvacservices.com</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>https://planohvacservices.com/local/richardson-heat-pump-installation.html</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr"/>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>info@planohvacservices.com</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>(469) 526-5070</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>Richardson TX</t>
+        </is>
+      </c>
+      <c r="I245" t="n">
+        <v>84</v>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>heat pump installation Richardson TX</t>
+        </is>
+      </c>
+      <c r="K245" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 19:07 UTC (cycle 19)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L245"/>
+  <dimension ref="A1:L246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -14669,7 +14669,6 @@
           <t>https://planohvacservices.com/local/richardson-heat-pump-installation.html</t>
         </is>
       </c>
-      <c r="E245" t="inlineStr"/>
       <c r="F245" t="inlineStr">
         <is>
           <t>info@planohvacservices.com</t>
@@ -14699,6 +14698,66 @@
         </is>
       </c>
       <c r="L245" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Air Conditioning Installation in Palm Bay FL | Quality Comfort</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>qualitycomfortfl.com</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>https://www.qualitycomfortfl.com/service-locations/palm-bay-florida-service-area/23-air-conditioning-installation-in-palm-bay-fl-quality-comfort.html</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Palm Bay</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>info@qualitycomfortfl.com</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>321-242-2513</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="I246" t="n">
+        <v>84</v>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>AC installation Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="K246" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L246" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 19:16 UTC (cycle 25)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L246"/>
+  <dimension ref="A1:L247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -14763,6 +14763,62 @@
         </is>
       </c>
     </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Plumbing Services in Fontana, CA | RN Plumbing &amp; Rooter</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>rnplumbingandrooter.com</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>https://rnplumbingandrooter.com/service-areas/fontana-ca</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr"/>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>rn.sonsconstructioninc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>9097611113</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>Fontana CA</t>
+        </is>
+      </c>
+      <c r="I247" t="n">
+        <v>90</v>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>plumbing company Fontana CA</t>
+        </is>
+      </c>
+      <c r="K247" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L247" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 19:18 UTC (cycle 27)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L247"/>
+  <dimension ref="A1:L248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -14784,7 +14784,6 @@
           <t>https://rnplumbingandrooter.com/service-areas/fontana-ca</t>
         </is>
       </c>
-      <c r="E247" t="inlineStr"/>
       <c r="F247" t="inlineStr">
         <is>
           <t>rn.sonsconstructioninc@gmail.com</t>
@@ -14814,6 +14813,66 @@
         </is>
       </c>
       <c r="L247" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>FiveStar Plumbing</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>fivestarplumbingcompany.com</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>https://fivestarplumbingcompany.com/sewers-and-drains/sewer-repairs-replacements/</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Head Supervisor</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>service@fivestarbuilding.net</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>(615) 382-8131</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>Nashville TN</t>
+        </is>
+      </c>
+      <c r="I248" t="n">
+        <v>90</v>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>sewer repair Nashville TN</t>
+        </is>
+      </c>
+      <c r="K248" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L248" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 19:21 UTC (cycle 29)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L248"/>
+  <dimension ref="A1:L251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -14878,6 +14878,182 @@
         </is>
       </c>
     </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Plumber Experts | North Wind Plumbing LLC  | Evansville, IN</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>northwindplumbingllc.com</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>https://www.northwindplumbingllc.com/</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr"/>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>northwindplumbingllc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>(812) 483-3977</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>Evansville IN</t>
+        </is>
+      </c>
+      <c r="I249" t="n">
+        <v>90</v>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>plumber Evansville IN</t>
+        </is>
+      </c>
+      <c r="K249" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L249" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>AC Heroes Manatee and Sarasota Country</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>ac-heroes.com</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>https://ac-heroes.com/</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>Manatee County</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>zach@ac-heroes.com</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>(941) 724-7127</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>Sarasota FL</t>
+        </is>
+      </c>
+      <c r="I250" t="n">
+        <v>90</v>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>AC installation Sarasota FL</t>
+        </is>
+      </c>
+      <c r="K250" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Keepin You Kool</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>keepinyoukool.com</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>https://keepinyoukool.com/services/ac-replacements-installations-sarasota/</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Residential Air</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>marc.bryant@keepinyoukool.com</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>(941) 448-1644</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>Sarasota FL</t>
+        </is>
+      </c>
+      <c r="I251" t="n">
+        <v>90</v>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>AC installation Sarasota FL</t>
+        </is>
+      </c>
+      <c r="K251" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 19:23 UTC (cycle 30)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L251"/>
+  <dimension ref="A1:L252"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -14899,7 +14899,6 @@
           <t>https://www.northwindplumbingllc.com/</t>
         </is>
       </c>
-      <c r="E249" t="inlineStr"/>
       <c r="F249" t="inlineStr">
         <is>
           <t>northwindplumbingllc@gmail.com</t>
@@ -15049,6 +15048,66 @@
         </is>
       </c>
       <c r="L251" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Performance Roofing of Colorado</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>performanceroofingco.com</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>https://performanceroofingco.com/service-areas/thornton/</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Community Preference</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>sales@performancegroupco.com</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>(720) 202-2000</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>Thornton CO</t>
+        </is>
+      </c>
+      <c r="I252" t="n">
+        <v>100</v>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>roofer Thornton CO</t>
+        </is>
+      </c>
+      <c r="K252" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L252" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 19:30 UTC (cycle 35)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L252"/>
+  <dimension ref="A1:L253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -15113,6 +15113,62 @@
         </is>
       </c>
     </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Sewer Line Repair | Elgin, IL | Ganziano Sewer &amp; Water</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>ganzianoseweril.com</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>https://www.ganzianoseweril.com/contact/sewer-line-repair-service-area/elgin-il</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr"/>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>joe@ganzianosewer.com</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>(847) 250-0904</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>Elgin IL</t>
+        </is>
+      </c>
+      <c r="I253" t="n">
+        <v>94</v>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>sewer repair Elgin IL</t>
+        </is>
+      </c>
+      <c r="K253" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 19:33 UTC (cycle 37)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L253"/>
+  <dimension ref="A1:L254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -15134,7 +15134,6 @@
           <t>https://www.ganzianoseweril.com/contact/sewer-line-repair-service-area/elgin-il</t>
         </is>
       </c>
-      <c r="E253" t="inlineStr"/>
       <c r="F253" t="inlineStr">
         <is>
           <t>joe@ganzianosewer.com</t>
@@ -15164,6 +15163,62 @@
         </is>
       </c>
       <c r="L253" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Portland Air Conditioning &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>portlandairconditioningheating.com</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>https://www.portlandairconditioningheating.com/</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr"/>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>info@portlandairconditioningheating.com</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>(971) 484-4490</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>Portland OR</t>
+        </is>
+      </c>
+      <c r="I254" t="n">
+        <v>90</v>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>air conditioning repair Portland OR</t>
+        </is>
+      </c>
+      <c r="K254" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L254" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 19:38 UTC (cycle 40)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L254"/>
+  <dimension ref="A1:L255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -15189,7 +15189,6 @@
           <t>https://www.portlandairconditioningheating.com/</t>
         </is>
       </c>
-      <c r="E254" t="inlineStr"/>
       <c r="F254" t="inlineStr">
         <is>
           <t>info@portlandairconditioningheating.com</t>
@@ -15219,6 +15218,66 @@
         </is>
       </c>
       <c r="L254" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Air Conditioning Service and Repair El Paso TX</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>totalairep.com</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>https://www.totalairep.com/</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Brandon Brooks</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>totalairsales@gmail.com</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>915-585-0909</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>El Paso TX</t>
+        </is>
+      </c>
+      <c r="I255" t="n">
+        <v>100</v>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>air conditioning repair El Paso TX</t>
+        </is>
+      </c>
+      <c r="K255" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L255" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 19:39 UTC (cycle 41)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L255"/>
+  <dimension ref="A1:L256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -15283,6 +15283,62 @@
         </is>
       </c>
     </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Elevated Plumbing</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>elevatedphcidaho.com</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>https://elevatedphcidaho.com/plumbers-in-nampa-idaho/</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr"/>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>epofidaho@gmail.com</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>(208) 615-7320</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>Nampa ID</t>
+        </is>
+      </c>
+      <c r="I256" t="n">
+        <v>100</v>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>plumbing company Nampa ID</t>
+        </is>
+      </c>
+      <c r="K256" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 19:41 UTC (cycle 42)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L256"/>
+  <dimension ref="A1:L257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -15304,7 +15304,6 @@
           <t>https://elevatedphcidaho.com/plumbers-in-nampa-idaho/</t>
         </is>
       </c>
-      <c r="E256" t="inlineStr"/>
       <c r="F256" t="inlineStr">
         <is>
           <t>epofidaho@gmail.com</t>
@@ -15334,6 +15333,66 @@
         </is>
       </c>
       <c r="L256" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>wordpress-1501121-6106766.cloudwaysapps.com</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>chucktownplumbing.com</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>https://chucktownplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Pleasant Plumbing</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>merissaferraraelisei@gmail.com</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>(843) 303-9364</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>Mount Pleasant SC</t>
+        </is>
+      </c>
+      <c r="I257" t="n">
+        <v>100</v>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>plumber Mount Pleasant SC</t>
+        </is>
+      </c>
+      <c r="K257" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L257" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 19:45 UTC (cycle 45)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L257"/>
+  <dimension ref="A1:L258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -15398,6 +15398,66 @@
         </is>
       </c>
     </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Plumber in Orange County | 24/7 Repair | SoCal Plumbing Co</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>socalplumbingco.com</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>https://socalplumbingco.com/services/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Home About</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>info@socalplumbingco.com</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>(562) 366-0303</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>Irvine CA</t>
+        </is>
+      </c>
+      <c r="I258" t="n">
+        <v>90</v>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>drain cleaning service Irvine CA</t>
+        </is>
+      </c>
+      <c r="K258" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 19:51 UTC (cycle 49)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L258"/>
+  <dimension ref="A1:L261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -15458,6 +15458,178 @@
         </is>
       </c>
     </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Anchor Exteriors KC</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>anchorexteriorskc.com</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>https://www.anchorexteriorskc.com/locations/lees-summit</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Anchor Exteriors</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>info@anchorexteriorskc.com</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>816-589-8629</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>Lees Summit MO</t>
+        </is>
+      </c>
+      <c r="I259" t="n">
+        <v>90</v>
+      </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>roofing contractor Lees Summit MO</t>
+        </is>
+      </c>
+      <c r="K259" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L259" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Metal Roof Springfield MO</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>metalroofspringfieldmo.com</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>http://metalroofspringfieldmo.com/</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr"/>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>moreinfo@metalroofspringfieldmo.com</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>866-868-1006</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>Springfield MO</t>
+        </is>
+      </c>
+      <c r="I260" t="n">
+        <v>84</v>
+      </c>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Springfield MO</t>
+        </is>
+      </c>
+      <c r="K260" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L260" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Roofing Contractor Springfield MO specializing in steel roofing installation | J</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>johnsonsroofingmo.com</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>https://www.johnsonsroofingmo.com/metal-roof-installation</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr"/>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>johnsonsroofingllc22@gmail.com</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>417-834-5050</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>Springfield MO</t>
+        </is>
+      </c>
+      <c r="I261" t="n">
+        <v>84</v>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Springfield MO</t>
+        </is>
+      </c>
+      <c r="K261" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 19:54 UTC (cycle 51)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L261"/>
+  <dimension ref="A1:L262"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -15539,7 +15539,6 @@
           <t>http://metalroofspringfieldmo.com/</t>
         </is>
       </c>
-      <c r="E260" t="inlineStr"/>
       <c r="F260" t="inlineStr">
         <is>
           <t>moreinfo@metalroofspringfieldmo.com</t>
@@ -15595,7 +15594,6 @@
           <t>https://www.johnsonsroofingmo.com/metal-roof-installation</t>
         </is>
       </c>
-      <c r="E261" t="inlineStr"/>
       <c r="F261" t="inlineStr">
         <is>
           <t>johnsonsroofingllc22@gmail.com</t>
@@ -15625,6 +15623,66 @@
         </is>
       </c>
       <c r="L261" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Starka Home</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>starkahome.com</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>https://www.starkahome.com/service-areas/pocatello</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Starka Home</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>info@starkahome.com</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>(509) 509-0161</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>Pocatello ID</t>
+        </is>
+      </c>
+      <c r="I262" t="n">
+        <v>90</v>
+      </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>roofing contractor Pocatello ID</t>
+        </is>
+      </c>
+      <c r="K262" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L262" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 19:59 UTC (cycle 54)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L262"/>
+  <dimension ref="A1:L263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -15688,6 +15688,66 @@
         </is>
       </c>
     </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Lakewood Drain Cleaning</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>lakewooddraincleaning.com</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>https://lakewooddraincleaning.com/</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Why Choose</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>info@lakewooddrainsolutions.com</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>(607) 558-1580</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>Lakewood CO</t>
+        </is>
+      </c>
+      <c r="I263" t="n">
+        <v>84</v>
+      </c>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>drain cleaning service Lakewood CO</t>
+        </is>
+      </c>
+      <c r="K263" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 20:06 UTC (cycle 59)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L263"/>
+  <dimension ref="A1:L265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -15748,6 +15748,126 @@
         </is>
       </c>
     </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Optimus Plumbing and Repair</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>optimusplumbingtn.com</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>https://www.optimusplumbingtn.com/johnson-city-tn/</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Johnson City</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>optimusplumbingandrepair@gmail.com</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>(423) 483-3777</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>Johnson City TN</t>
+        </is>
+      </c>
+      <c r="I264" t="n">
+        <v>100</v>
+      </c>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>sewer repair Johnson City TN</t>
+        </is>
+      </c>
+      <c r="K264" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L264" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Klaus and Sons</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>klausandsons.com</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>https://klausandsons.com/service-area/rancho-cucamonga-ca-plumbing-heating-air-conditioning/</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Allison Sachs</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>heather@klausandsons.com</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>909-982-5698</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>Rancho Cucamonga CA</t>
+        </is>
+      </c>
+      <c r="I265" t="n">
+        <v>90</v>
+      </c>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>HVAC contractor Rancho Cucamonga CA</t>
+        </is>
+      </c>
+      <c r="K265" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L265" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 20:09 UTC (cycle 61)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L265"/>
+  <dimension ref="A1:L268"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -15868,6 +15868,186 @@
         </is>
       </c>
     </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>AC Repairs by ColdHVAC</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>acrepairsbycoldhvac.com</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>https://acrepairsbycoldhvac.com/hvac-in-hialeah-fl/</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Team The</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>info@acrepairsbycoldhvac.com</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>(645) 238-2941</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>Hialeah FL</t>
+        </is>
+      </c>
+      <c r="I266" t="n">
+        <v>90</v>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>HVAC contractor Hialeah FL</t>
+        </is>
+      </c>
+      <c r="K266" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L266" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>AmazingCold AC Repairs</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>amazingcoldacrepairs.com</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>https://amazingcoldacrepairs.com/</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Team The</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>info@amazingcoldacrepairs.com</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>(786) 224-3314</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>Hialeah FL</t>
+        </is>
+      </c>
+      <c r="I267" t="n">
+        <v>90</v>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>HVAC contractor Hialeah FL</t>
+        </is>
+      </c>
+      <c r="K267" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L267" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>MaxHVAC Air Conditioning Repair</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>maxhvacacrepair.com</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>https://maxhvacacrepair.com/hvac-in-hialeah-fl/</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Team The</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>info@maxhvacacrepair.com</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>(305) 280-5794</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>Hialeah FL</t>
+        </is>
+      </c>
+      <c r="I268" t="n">
+        <v>90</v>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>HVAC contractor Hialeah FL</t>
+        </is>
+      </c>
+      <c r="K268" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 20:21 UTC (cycle 69)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L268"/>
+  <dimension ref="A1:L269"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -16048,6 +16048,66 @@
         </is>
       </c>
     </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Newman's Plumbing Service &amp; Repair</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>newmansplumbingservice.com</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>https://www.newmansplumbingservice.com/service-areas/norfolk-va</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Why Choose</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>newmansplumbingservice@gmail.com</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>(757) 465-0883</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>Norfolk VA</t>
+        </is>
+      </c>
+      <c r="I269" t="n">
+        <v>100</v>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>sewer repair Norfolk VA</t>
+        </is>
+      </c>
+      <c r="K269" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L269" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 20:22 UTC (cycle 70)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L269"/>
+  <dimension ref="A1:L270"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -16108,6 +16108,66 @@
         </is>
       </c>
     </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Complete Temperature Services</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>completetemp.com</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>https://completetemp.com/</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Light Commercial</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>charlesgoldsmith@completetemp.com</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>(702) 488-8338</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>North Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="I270" t="n">
+        <v>98</v>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>HVAC contractor North Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="K270" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L270" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 20:32 UTC (cycle 77)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L270"/>
+  <dimension ref="A1:L272"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -16168,6 +16168,122 @@
         </is>
       </c>
     </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Mainline Plumbing, AC &amp; Electrical</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>mainlineplumbingservice.com</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>https://mainlineplumbingservice.com/service-area/coral-springs-fl/</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Serving Homeowners</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>info@mainlineplumbingservice.com</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>(954) 280-5597</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="I271" t="n">
+        <v>94</v>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>plumbing company Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="K271" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>High Level Plumbing</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>highlevelplumbingfl.com</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>https://www.highlevelplumbingfl.com/broward-county/coral-springs/</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr"/>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>bbarrancos@dharmamarketing.cloud</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>(786) 473-4124</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="I272" t="n">
+        <v>90</v>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>plumbing company Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 20:34 UTC (cycle 78)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L272"/>
+  <dimension ref="A1:L273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -16249,7 +16249,6 @@
           <t>https://www.highlevelplumbingfl.com/broward-county/coral-springs/</t>
         </is>
       </c>
-      <c r="E272" t="inlineStr"/>
       <c r="F272" t="inlineStr">
         <is>
           <t>bbarrancos@dharmamarketing.cloud</t>
@@ -16279,6 +16278,66 @@
         </is>
       </c>
       <c r="L272" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Nero's Heating And Air</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>neroshvac.com</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>https://neroshvac.com/hvac-in-germantown-md/</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Virginia Northern</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>info@neroshvac.com</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>(202) 750-9543</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>Germantown MD</t>
+        </is>
+      </c>
+      <c r="I273" t="n">
+        <v>90</v>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>heating and cooling company Germantown MD</t>
+        </is>
+      </c>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L273" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 20:38 UTC (cycle 81)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L273"/>
+  <dimension ref="A1:L275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -16343,6 +16343,126 @@
         </is>
       </c>
     </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Done Right Roofing</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>donerightroofingva.com</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>https://donerightroofingva.com/chesapeake-va/</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Newport News</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>lbdconstructions757@gmail.com</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>(757) 553-4048</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>Chesapeake VA</t>
+        </is>
+      </c>
+      <c r="I274" t="n">
+        <v>100</v>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>roof replacement Chesapeake VA</t>
+        </is>
+      </c>
+      <c r="K274" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Benoure Plumbing, Heating &amp; Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>benoure.com</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>https://www.benoure.com/hvac-plumbing-service/</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Follow Careers</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>info@benoure.com</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>802-864-7156</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>Burlington VT</t>
+        </is>
+      </c>
+      <c r="I275" t="n">
+        <v>100</v>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>air conditioning repair Burlington VT</t>
+        </is>
+      </c>
+      <c r="K275" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 20:54 UTC (cycle 92)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L275"/>
+  <dimension ref="A1:L277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -16463,6 +16463,122 @@
         </is>
       </c>
     </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Hargrave's Plumbing, LLC</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>hargravesplumbing.com</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>https://www.hargravesplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr"/>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>travis@hargravesplumbing.com</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>337-344-3920</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>Lafayette LA</t>
+        </is>
+      </c>
+      <c r="I276" t="n">
+        <v>90</v>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>plumber Lafayette LA</t>
+        </is>
+      </c>
+      <c r="K276" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Roofing Repair &amp; Replacement in Juneau, AK</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>glacierbearconstruction.com</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>https://www.glacierbearconstruction.com/exterior/roofing</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Kinnon Scharen</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>kscharen@glacierbearconstruction.com</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>(907) 635-0756</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>Juneau AK</t>
+        </is>
+      </c>
+      <c r="I277" t="n">
+        <v>90</v>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>roof repair company Juneau AK</t>
+        </is>
+      </c>
+      <c r="K277" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 21:07 UTC (cycle 101)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L277"/>
+  <dimension ref="A1:L278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -16484,7 +16484,6 @@
           <t>https://www.hargravesplumbing.com/</t>
         </is>
       </c>
-      <c r="E276" t="inlineStr"/>
       <c r="F276" t="inlineStr">
         <is>
           <t>travis@hargravesplumbing.com</t>
@@ -16574,6 +16573,66 @@
         </is>
       </c>
       <c r="L277" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Bayfront Roofing and Construction</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>bayfrontroofing.com</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>https://bayfrontroofing.com/</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Corpus Christi</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>bestroofers@bayfrontroofing.com</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>(361) 800-5991</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="I278" t="n">
+        <v>100</v>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>roofing contractor Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="K278" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L278" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 21:12 UTC (cycle 104)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L278"/>
+  <dimension ref="A1:L279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -16638,6 +16638,66 @@
         </is>
       </c>
     </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Steve's 5 Star Service</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>stevesair.com</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>https://www.stevesair.com/hvac-services-fontana.php</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Inland Empire</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>office@stevesair.com</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>(909) 985-5254</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>Fontana CA</t>
+        </is>
+      </c>
+      <c r="I279" t="n">
+        <v>90</v>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>heating and cooling company Fontana CA</t>
+        </is>
+      </c>
+      <c r="K279" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 21:22 UTC (cycle 111)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L279"/>
+  <dimension ref="A1:L280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -16698,6 +16698,66 @@
         </is>
       </c>
     </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>DHT Construction &amp; Roofing</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>dhtconstructionwa.com</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>https://dhtconstructionwa.com/</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Protecting Tacoma</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>curtis.dht@gmail.com</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>(253) 367-2774</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>Tacoma WA</t>
+        </is>
+      </c>
+      <c r="I280" t="n">
+        <v>80</v>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>roof repair company Tacoma WA</t>
+        </is>
+      </c>
+      <c r="K280" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 21:25 UTC (cycle 113)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L280"/>
+  <dimension ref="A1:L281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -16758,6 +16758,62 @@
         </is>
       </c>
     </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>New Haven Furnace Repair In Your Area</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>newhavenhvac.net</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>https://newhavenhvac.net/new-haven-furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr"/>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>service@newhavenhvac.net</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>844-731-1625</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>New Haven CT</t>
+        </is>
+      </c>
+      <c r="I281" t="n">
+        <v>90</v>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>furnace repair New Haven CT</t>
+        </is>
+      </c>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 21:26 UTC (cycle 114)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L281"/>
+  <dimension ref="A1:L283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -16779,7 +16779,6 @@
           <t>https://newhavenhvac.net/new-haven-furnace-repair/</t>
         </is>
       </c>
-      <c r="E281" t="inlineStr"/>
       <c r="F281" t="inlineStr">
         <is>
           <t>service@newhavenhvac.net</t>
@@ -16809,6 +16808,122 @@
         </is>
       </c>
       <c r="L281" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Antebellum Roofworks</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>antebellumroofworks.com</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>https://antebellumroofworks.com/franklin-tn/</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Caps Cupolas</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>info@antebellumroofworks.com</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>(615) 794-9111</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>Franklin TN</t>
+        </is>
+      </c>
+      <c r="I282" t="n">
+        <v>100</v>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>residential roofing company Franklin TN</t>
+        </is>
+      </c>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>Pine Knot Roofing</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>pineknotroofing.com</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>https://pineknotroofing.com/residential-roofing-company-in-franklin-tn/</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Dustin Sullivan</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>info@pineknotroofing.com</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr"/>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>Franklin TN</t>
+        </is>
+      </c>
+      <c r="I283" t="n">
+        <v>76</v>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>residential roofing company Franklin TN</t>
+        </is>
+      </c>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L283" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 21:28 UTC (cycle 115)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L283"/>
+  <dimension ref="A1:L284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -16904,7 +16904,6 @@
           <t>info@pineknotroofing.com</t>
         </is>
       </c>
-      <c r="G283" t="inlineStr"/>
       <c r="H283" t="inlineStr">
         <is>
           <t>Franklin TN</t>
@@ -16924,6 +16923,66 @@
         </is>
       </c>
       <c r="L283" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2nd Wind HVAC - Serving the communities in the Columbia, SC area since 1985</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>2ndwindhvac.com</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>https://2ndwindhvac.com/services/heating-columbia-sc/heat-pumps/</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>How We</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>service@2ndwindhvac.com</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>(803) 392-1513</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>Columbia SC</t>
+        </is>
+      </c>
+      <c r="I284" t="n">
+        <v>90</v>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>heat pump installation Columbia SC</t>
+        </is>
+      </c>
+      <c r="K284" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L284" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 21:29 UTC (cycle 116)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L284"/>
+  <dimension ref="A1:L288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -16988,6 +16988,242 @@
         </is>
       </c>
     </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>HVAC Services | McCormack Heating &amp; Cooling Inc | Huntsville, AL</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>mccormackheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>https://www.mccormackheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr"/>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>mccormackheatingandcooling@msn.com</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>(256) 533-2678</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>Huntsville AL</t>
+        </is>
+      </c>
+      <c r="I285" t="n">
+        <v>100</v>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>furnace repair Huntsville AL</t>
+        </is>
+      </c>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Air Repair AL</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>airrepairal.com</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>https://www.airrepairal.com/service-area/hvac-services-huntsville-al/</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Don Johnson</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>al@airrepairal.com</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>864-777-1111</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>Huntsville AL</t>
+        </is>
+      </c>
+      <c r="I286" t="n">
+        <v>100</v>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>furnace repair Huntsville AL</t>
+        </is>
+      </c>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>Bellevue Roofing Company, Inc</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>bellevueroofinginc.com</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>https://www.bellevueroofinginc.com/pages/services/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Bellevue Roofing</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>bellevueroofing@msn.com</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>(425)746-9867</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>Bellevue WA</t>
+        </is>
+      </c>
+      <c r="I287" t="n">
+        <v>90</v>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Bellevue WA</t>
+        </is>
+      </c>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Metal Roofing Bellevue WA | Accelerate Builder</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>acceleratebuilder.com</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>https://acceleratebuilder.com/metal-roofing-bellevue-wa</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Accelerate Builder</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>admin@acceleratebuilder.com</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>425-675-1592</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>Bellevue WA</t>
+        </is>
+      </c>
+      <c r="I288" t="n">
+        <v>88</v>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Bellevue WA</t>
+        </is>
+      </c>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 21:31 UTC (cycle 117)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L288"/>
+  <dimension ref="A1:L289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -17009,7 +17009,6 @@
           <t>https://www.mccormackheatingandcooling.com/</t>
         </is>
       </c>
-      <c r="E285" t="inlineStr"/>
       <c r="F285" t="inlineStr">
         <is>
           <t>mccormackheatingandcooling@msn.com</t>
@@ -17219,6 +17218,66 @@
         </is>
       </c>
       <c r="L288" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>Essential Peak Roofing</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>essentialpeakroofinginc.com</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>https://essentialpeakroofinginc.com/roofing-contractor-elk-grove-ca/</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Northern California</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>essentialpeakroofinginc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>(279) 269-3331</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>Elk Grove CA</t>
+        </is>
+      </c>
+      <c r="I289" t="n">
+        <v>90</v>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>roofing contractor Elk Grove CA</t>
+        </is>
+      </c>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L289" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 21:37 UTC (cycle 121)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L289"/>
+  <dimension ref="A1:L290"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -17283,6 +17283,66 @@
         </is>
       </c>
     </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>Roofer Lakeland Fl</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>rooferlakelandfl.com</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>https://rooferlakelandfl.com/</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Projects Completed</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>info@rooferlakelandfl.com</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>(844) 907-2549</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>Lakeland FL</t>
+        </is>
+      </c>
+      <c r="I290" t="n">
+        <v>90</v>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>roofer Lakeland FL</t>
+        </is>
+      </c>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 21:41 UTC (cycle 124)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L290"/>
+  <dimension ref="A1:L291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -17343,6 +17343,66 @@
         </is>
       </c>
     </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Roof Replacement Westminster, CO | Weaver Construction USA</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>weaverconstructionusa.com</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>https://www.weaverconstructionusa.com/service-areas/westminster-co/roof-replacement</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Weaver Construction</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>info@weaverconstructionusa.com</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>(720) 314-6777</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>Westminster CO</t>
+        </is>
+      </c>
+      <c r="I291" t="n">
+        <v>90</v>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>roof replacement Westminster CO</t>
+        </is>
+      </c>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 21:43 UTC (cycle 125)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L291"/>
+  <dimension ref="A1:L293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -17403,6 +17403,118 @@
         </is>
       </c>
     </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Drain Cleaners | Elgin, IL | ASAP Plumbing</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>asapplumbingnow.com</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>https://www.asapplumbingnow.com/contact/drain-cleaners-service-area/elgin-il</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr"/>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>info@asapplumbing.org</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>(815) 201-2940</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>Elgin IL</t>
+        </is>
+      </c>
+      <c r="I292" t="n">
+        <v>100</v>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>drain cleaning service Elgin IL</t>
+        </is>
+      </c>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>WeatherPro Exteriors</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>weatherproexteriors.com</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>https://www.weatherproexteriors.com/Wisconsin/Waukesha</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr"/>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>info@weatherproexteriors.com</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>(414) 543-0929</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>Waukesha WI</t>
+        </is>
+      </c>
+      <c r="I293" t="n">
+        <v>100</v>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>roofing contractor Waukesha WI</t>
+        </is>
+      </c>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 21:44 UTC (cycle 126)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L293"/>
+  <dimension ref="A1:L294"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -17424,7 +17424,6 @@
           <t>https://www.asapplumbingnow.com/contact/drain-cleaners-service-area/elgin-il</t>
         </is>
       </c>
-      <c r="E292" t="inlineStr"/>
       <c r="F292" t="inlineStr">
         <is>
           <t>info@asapplumbing.org</t>
@@ -17480,7 +17479,6 @@
           <t>https://www.weatherproexteriors.com/Wisconsin/Waukesha</t>
         </is>
       </c>
-      <c r="E293" t="inlineStr"/>
       <c r="F293" t="inlineStr">
         <is>
           <t>info@weatherproexteriors.com</t>
@@ -17510,6 +17508,66 @@
         </is>
       </c>
       <c r="L293" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Residential Roofing Services | San Francisco, CA | Anderson Roofing &amp; Sheet Meta</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>andersonroofingcompany.com</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>https://www.andersonroofingcompany.com/residential-roofing-services</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>andersonroofingsf@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>415-584-9575</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>San Francisco CA</t>
+        </is>
+      </c>
+      <c r="I294" t="n">
+        <v>84</v>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>residential roofing company San Francisco CA</t>
+        </is>
+      </c>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L294" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 21:46 UTC (cycle 127)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L294"/>
+  <dimension ref="A1:L295"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -17573,6 +17573,62 @@
         </is>
       </c>
     </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Madison Plumbing Pros | Licensed Plumbers in Madison, WI</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>madisonplumbingpros.com</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>https://madisonplumbingpros.com/</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Dane County</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>contact@madisonplumbingpros.com</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr"/>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>Madison WI</t>
+        </is>
+      </c>
+      <c r="I295" t="n">
+        <v>86</v>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>plumbing company Madison WI</t>
+        </is>
+      </c>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 21:47 UTC (cycle 128)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L295"/>
+  <dimension ref="A1:L298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -17604,7 +17604,6 @@
           <t>contact@madisonplumbingpros.com</t>
         </is>
       </c>
-      <c r="G295" t="inlineStr"/>
       <c r="H295" t="inlineStr">
         <is>
           <t>Madison WI</t>
@@ -17624,6 +17623,186 @@
         </is>
       </c>
       <c r="L295" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Eagle Pro Heating, Cooling, Plumbing &amp; Insulation</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>calleaglepro.com</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>https://calleaglepro.com/service-area/huntsville-al/ac-installation/</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>North Alabama</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>info@eagleprollc.com</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>256-767-5154</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>Huntsville AL</t>
+        </is>
+      </c>
+      <c r="I296" t="n">
+        <v>100</v>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>AC installation Huntsville AL</t>
+        </is>
+      </c>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Oregon Exterior Experts</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>oregonexteriorexperts.com</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>https://oregonexteriorexperts.com/roofing/replacement/beaverton/</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Lake Oswego</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>admin@oregonexteriorexperts.com</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>(971) 217-7402</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>Beaverton OR</t>
+        </is>
+      </c>
+      <c r="I297" t="n">
+        <v>96</v>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>roof replacement Beaverton OR</t>
+        </is>
+      </c>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>HVAC, Plumbing, and Electrical Services</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>callmpe.com</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>https://www.callmpe.com/ac-installation-huntsville-al</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Generators Whole</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>service@callmpe.com</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>256-766-9439</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>Huntsville AL</t>
+        </is>
+      </c>
+      <c r="I298" t="n">
+        <v>80</v>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>AC installation Huntsville AL</t>
+        </is>
+      </c>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L298" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 21:56 UTC (cycle 134)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L298"/>
+  <dimension ref="A1:L299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -17808,6 +17808,66 @@
         </is>
       </c>
     </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Providence Plumbing</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>providenceplumbling.com</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>https://providenceplumbling.com/</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Westminster St</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>info@providenceplumbling.com</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>(401) 394 4927</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>Providence RI</t>
+        </is>
+      </c>
+      <c r="I299" t="n">
+        <v>100</v>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>emergency plumber Providence RI</t>
+        </is>
+      </c>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 22:02 UTC (cycle 138)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L299"/>
+  <dimension ref="A1:L300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -17868,6 +17868,66 @@
         </is>
       </c>
     </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Connected Air Conditioning &amp; Heating Repair</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>connectedheatingandairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>https://connectedheatingandairconditioning.com/locations/elizabeth-nj.html</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Most Elizabeth</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>service@connectedheatingandairconditioning.com</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>(877) 493-8217</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>Elizabeth NJ</t>
+        </is>
+      </c>
+      <c r="I300" t="n">
+        <v>90</v>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>furnace repair Elizabeth NJ</t>
+        </is>
+      </c>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 22:03 UTC (cycle 139)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L300"/>
+  <dimension ref="A1:L302"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -17928,6 +17928,122 @@
         </is>
       </c>
     </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Druziako HVAC</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>druziakohvac.com</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>https://druziakohvac.com/</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr"/>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>office@druziakohvac.com</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>978-441-9800</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>Lowell MA</t>
+        </is>
+      </c>
+      <c r="I301" t="n">
+        <v>100</v>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>AC installation Lowell MA</t>
+        </is>
+      </c>
+      <c r="K301" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>HVAC Services in Woodbridge, NJ</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>richshvacexperts.com</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>https://richshvacexperts.com/service-areas/hvac-services-in-woodbridge-nj/</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Central New</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>info@richshvacexperts.com</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>(732) 433-0068</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>Woodbridge NJ</t>
+        </is>
+      </c>
+      <c r="I302" t="n">
+        <v>100</v>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>heating and cooling company Woodbridge NJ</t>
+        </is>
+      </c>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 22:06 UTC (cycle 141)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L302"/>
+  <dimension ref="A1:L303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -17949,7 +17949,6 @@
           <t>https://druziakohvac.com/</t>
         </is>
       </c>
-      <c r="E301" t="inlineStr"/>
       <c r="F301" t="inlineStr">
         <is>
           <t>office@druziakohvac.com</t>
@@ -18039,6 +18038,66 @@
         </is>
       </c>
       <c r="L302" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Hialeah Drain Cleaning</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>hialeahdraincleaning.com</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>https://hialeahdraincleaning.com/</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>Hialeah Homeowners</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>info@hialeahdraincleaning.com</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>(855) 734-3235</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>Hialeah FL</t>
+        </is>
+      </c>
+      <c r="I303" t="n">
+        <v>84</v>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>drain cleaning service Hialeah FL</t>
+        </is>
+      </c>
+      <c r="K303" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L303" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 22:09 UTC (cycle 143)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L303"/>
+  <dimension ref="A1:L304"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -18103,6 +18103,62 @@
         </is>
       </c>
     </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Air Conditioning Installation Laredo, TX.</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>expressaircooling.com</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>https://expressaircooling.com/areas-of-service/air-conditioning-installation-laredo/</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr"/>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>expressairac@gmail.com</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>(956) 722-2665</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>Laredo TX</t>
+        </is>
+      </c>
+      <c r="I304" t="n">
+        <v>90</v>
+      </c>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>AC installation Laredo TX</t>
+        </is>
+      </c>
+      <c r="K304" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 22:14 UTC (cycle 146)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L304"/>
+  <dimension ref="A1:L305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -18124,7 +18124,6 @@
           <t>https://expressaircooling.com/areas-of-service/air-conditioning-installation-laredo/</t>
         </is>
       </c>
-      <c r="E304" t="inlineStr"/>
       <c r="F304" t="inlineStr">
         <is>
           <t>expressairac@gmail.com</t>
@@ -18154,6 +18153,66 @@
         </is>
       </c>
       <c r="L304" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Honeycomb Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>honeycombair.com</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>https://honeycombair.com/service/cooling/ac-installation/</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>San Antonio</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>office@honeycombair.com</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>(726) 233-6044</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I305" t="n">
+        <v>100</v>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>AC installation New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K305" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L305" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 22:18 UTC (cycle 149)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L305"/>
+  <dimension ref="A1:L306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -18218,6 +18218,66 @@
         </is>
       </c>
     </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>C&amp;A Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>caroofingconstruction.com</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>https://www.caroofingconstruction.com/service-areas/broken-arrow</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>Trusted Contractor</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>info@caroofingconstruction.com</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>(918) 637-6634</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>Broken Arrow OK</t>
+        </is>
+      </c>
+      <c r="I306" t="n">
+        <v>86</v>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>roofer Broken Arrow OK</t>
+        </is>
+      </c>
+      <c r="K306" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 22:20 UTC (cycle 150)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L306"/>
+  <dimension ref="A1:L307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -18278,6 +18278,62 @@
         </is>
       </c>
     </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Browns Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>brownshvac.net</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>https://brownshvac.net/heating/water-heaters/water-heater-repair-chicago/</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr"/>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>support@brownshvac.net</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>(708) 536-8134</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>Chicago IL</t>
+        </is>
+      </c>
+      <c r="I307" t="n">
+        <v>100</v>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>water heater repair Chicago IL</t>
+        </is>
+      </c>
+      <c r="K307" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 22:30 UTC (cycle 157)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L307"/>
+  <dimension ref="A1:L308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -18299,7 +18299,6 @@
           <t>https://brownshvac.net/heating/water-heaters/water-heater-repair-chicago/</t>
         </is>
       </c>
-      <c r="E307" t="inlineStr"/>
       <c r="F307" t="inlineStr">
         <is>
           <t>support@brownshvac.net</t>
@@ -18329,6 +18328,66 @@
         </is>
       </c>
       <c r="L307" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>Temperature Solutions</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>tempsolutions.net</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>https://www.tempsolutions.net/services/hvac-contractor/air-conditioning-installation</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>Client Reviews</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>nick.collins@tempsolutions.net</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>(863) 430-3650</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>Lakeland FL</t>
+        </is>
+      </c>
+      <c r="I308" t="n">
+        <v>100</v>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>AC installation Lakeland FL</t>
+        </is>
+      </c>
+      <c r="K308" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L308" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 22:34 UTC (cycle 160)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L308"/>
+  <dimension ref="A1:L309"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -18393,6 +18393,66 @@
         </is>
       </c>
     </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Eddy Exteriors LLC</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>eddyexteriorsllc.com</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>https://www.eddyexteriorsllc.com/</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Start To</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>eddyexteriorsllc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>(517) 896-7591</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>Lansing MI</t>
+        </is>
+      </c>
+      <c r="I309" t="n">
+        <v>100</v>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>residential roofing company Lansing MI</t>
+        </is>
+      </c>
+      <c r="K309" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 22:55 UTC (cycle 174)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L309"/>
+  <dimension ref="A1:L310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -18453,6 +18453,62 @@
         </is>
       </c>
     </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>R Hvac</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>rrhvacservice.com</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>https://www.rrhvacservice.com/</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr"/>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>rrhvacservices.2025@gmail.com</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>585-545-0895</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>Rochester NY</t>
+        </is>
+      </c>
+      <c r="I310" t="n">
+        <v>88</v>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>HVAC contractor Rochester NY</t>
+        </is>
+      </c>
+      <c r="K310" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 23:05 UTC (cycle 181)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L310"/>
+  <dimension ref="A1:L313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -18474,7 +18474,6 @@
           <t>https://www.rrhvacservice.com/</t>
         </is>
       </c>
-      <c r="E310" t="inlineStr"/>
       <c r="F310" t="inlineStr">
         <is>
           <t>rrhvacservices.2025@gmail.com</t>
@@ -18504,6 +18503,186 @@
         </is>
       </c>
       <c r="L310" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>Merritt Roofing, INC.</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>merrittroofingpolk.com</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>https://merrittroofingpolk.com/lakeland-fl/</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>You Covered</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>merrittroofing@tampabay.rr.com</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>(863) 967-5711</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>Lakeland FL</t>
+        </is>
+      </c>
+      <c r="I311" t="n">
+        <v>100</v>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>roof repair company Lakeland FL</t>
+        </is>
+      </c>
+      <c r="K311" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L311" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Burnes Roofing Company, LLC - Owner-operated roofing contractor in Orlando, FL</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>burnesroofing.com</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>https://burnesroofing.com/roofing-lakeland-fl/</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Operated Orlando</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>burnesroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>407-446-9290</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>Lakeland FL</t>
+        </is>
+      </c>
+      <c r="I312" t="n">
+        <v>90</v>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>roof repair company Lakeland FL</t>
+        </is>
+      </c>
+      <c r="K312" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L312" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>High Tower Roofing</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>hightowerroofing.com</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>https://hightowerroofing.com/roof-repair-south-lakeland-fl/</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>Your Roof</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>contacthtr@hightowerroofing.com</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>863-510-5477</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>Lakeland FL</t>
+        </is>
+      </c>
+      <c r="I313" t="n">
+        <v>90</v>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>roof repair company Lakeland FL</t>
+        </is>
+      </c>
+      <c r="K313" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L313" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 23:08 UTC (cycle 183)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L313"/>
+  <dimension ref="A1:L315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -18688,6 +18688,122 @@
         </is>
       </c>
     </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>Freedom Restoration and Roofing</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>freedomroofingmo.com</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>https://freedomroofingmo.com/residential-roofing-st-charles-mo/</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>Roof Reviews</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>info@freedomroofingmo.com</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>(636) 498-4200</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>St Charles MO</t>
+        </is>
+      </c>
+      <c r="I314" t="n">
+        <v>90</v>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>residential roofing company St Charles MO</t>
+        </is>
+      </c>
+      <c r="K314" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L314" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>Right Choice Roofing | (636) 466-8964</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>rightchoiceroofingstl.com</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>https://rightchoiceroofingstl.com/residential-roofing-st-charles-mo/</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr"/>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>rightchoiceroofingstl@gmail.com</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>(636) 466-8964</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>St Charles MO</t>
+        </is>
+      </c>
+      <c r="I315" t="n">
+        <v>90</v>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>residential roofing company St Charles MO</t>
+        </is>
+      </c>
+      <c r="K315" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L315" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 23:14 UTC (cycle 187)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L315"/>
+  <dimension ref="A1:L317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -18769,7 +18769,6 @@
           <t>https://rightchoiceroofingstl.com/residential-roofing-st-charles-mo/</t>
         </is>
       </c>
-      <c r="E315" t="inlineStr"/>
       <c r="F315" t="inlineStr">
         <is>
           <t>rightchoiceroofingstl@gmail.com</t>
@@ -18799,6 +18798,122 @@
         </is>
       </c>
       <c r="L315" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>AMP Roofing &amp; Exteriors</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>amproofing.com</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>https://amproofing.com/metal-roofing-austin/</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>Roof Financing</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>website@amproofing.com</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>(512) 675-3323</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>Austin TX</t>
+        </is>
+      </c>
+      <c r="I316" t="n">
+        <v>100</v>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Austin TX</t>
+        </is>
+      </c>
+      <c r="K316" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L316" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>Kelley &amp; Dawson Service</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>kelleyanddawson.com</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>https://kelleyanddawson.com/heating/furnace-repair-service-wichita-ks</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr"/>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>info@kelleyanddawson.com</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>(316) 263-7201</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>Wichita KS</t>
+        </is>
+      </c>
+      <c r="I317" t="n">
+        <v>90</v>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>furnace repair Wichita KS</t>
+        </is>
+      </c>
+      <c r="K317" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L317" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 23:17 UTC (cycle 189)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L317"/>
+  <dimension ref="A1:L318"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -18884,7 +18884,6 @@
           <t>https://kelleyanddawson.com/heating/furnace-repair-service-wichita-ks</t>
         </is>
       </c>
-      <c r="E317" t="inlineStr"/>
       <c r="F317" t="inlineStr">
         <is>
           <t>info@kelleyanddawson.com</t>
@@ -18914,6 +18913,66 @@
         </is>
       </c>
       <c r="L317" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>DiMone Parlier Plumbing &amp; Irrigation</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>dimoneparlierplumbing.com</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>https://dimoneparlierplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>Internet Marketing</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>service@dimoneparlierplumbing.com</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>910-769-1838</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>Wilmington NC</t>
+        </is>
+      </c>
+      <c r="I318" t="n">
+        <v>100</v>
+      </c>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>plumbing company Wilmington NC</t>
+        </is>
+      </c>
+      <c r="K318" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L318" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 23:23 UTC (cycle 193)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L318"/>
+  <dimension ref="A1:L323"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -18978,6 +18978,306 @@
         </is>
       </c>
     </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>Pact Plumbing</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>pactplumbing.com</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>https://www.pactplumbing.com/plano-water-heater-repair/</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>Serving All</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>wade@pactplumbing.com</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>214-444-3697</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>Plano TX</t>
+        </is>
+      </c>
+      <c r="I319" t="n">
+        <v>100</v>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>water heater repair Plano TX</t>
+        </is>
+      </c>
+      <c r="K319" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L319" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>Plano TX Water Heater</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>planotxwaterheater.com</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>https://www.planotxwaterheater.com/</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>Safety And</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>service@planotxwaterheater.com</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>972-584-7301</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>Plano TX</t>
+        </is>
+      </c>
+      <c r="I320" t="n">
+        <v>100</v>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>water heater repair Plano TX</t>
+        </is>
+      </c>
+      <c r="K320" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L320" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>Water Heater Repair Plano TX</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>waterheaterrepairplano.com</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>https://waterheaterrepairplano.com/repair.html</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>Legacy West</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>service@waterheaterrepairplano.com</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>972-843-1326</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>Plano TX</t>
+        </is>
+      </c>
+      <c r="I321" t="n">
+        <v>94</v>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>water heater repair Plano TX</t>
+        </is>
+      </c>
+      <c r="K321" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L321" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>Roof Repair Houston</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>roofrepair.day</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>https://roofrepair.day/katy-metal-roofing</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>Fort Bend</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>office@roofrepair.day</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>(713) 936-5504</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>Katy TX</t>
+        </is>
+      </c>
+      <c r="I322" t="n">
+        <v>90</v>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Katy TX</t>
+        </is>
+      </c>
+      <c r="K322" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L322" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>Greiber Heating &amp; Sheet Metal</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>greiberheating.com</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>https://www.greiberheating.com/city/madison-wi/</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>Maintenance Plans</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>katie@greiberheating.com</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>(608) 795-3885</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>Madison WI</t>
+        </is>
+      </c>
+      <c r="I323" t="n">
+        <v>90</v>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>heating and cooling company Madison WI</t>
+        </is>
+      </c>
+      <c r="K323" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L323" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 23:26 UTC (cycle 195)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L323"/>
+  <dimension ref="A1:L325"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -19278,6 +19278,126 @@
         </is>
       </c>
     </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>Roofing Contractors in Sugar Land, Tx | Instant Estimates | New Roofs from $99/m</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>sugarroofs.com</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>https://www.sugarroofs.com/service-area/houston-tx/sugar-land-tx</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>Sugar Land</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>sales@sugarroofs.com</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>713-843-7204</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="I324" t="n">
+        <v>100</v>
+      </c>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>roofing contractor Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="K324" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L324" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Plumber Elite of Mount Vernon</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>plumberelitemountvernon.com</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>https://plumberelitemountvernon.com/</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>Plumber Elite</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>info@plumberelitemountvernon.com</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>(914)-221-5698</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="I325" t="n">
+        <v>90</v>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>plumbing company Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="K325" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L325" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 23:33 UTC (cycle 200)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L325"/>
+  <dimension ref="A1:L326"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -19398,6 +19398,66 @@
         </is>
       </c>
     </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>Metal Roofing, Residential and Commercial</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>smartroofers.com</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>https://www.smartroofers.com/Metal-Roofing.php</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>Metal Roofing</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>contactus@smartroofers.com</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>847.797.0404</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>Chicago IL</t>
+        </is>
+      </c>
+      <c r="I326" t="n">
+        <v>90</v>
+      </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Chicago IL</t>
+        </is>
+      </c>
+      <c r="K326" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L326" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 23:35 UTC (cycle 201)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L326"/>
+  <dimension ref="A1:L328"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -19458,6 +19458,126 @@
         </is>
       </c>
     </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>Sewell Service Company</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>sewellservicecompany.com</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>https://sewellservicecompany.com/</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>Birmingham Heating</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>marc@sitemaxmarketing.com</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>205-680-5066</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>Birmingham AL</t>
+        </is>
+      </c>
+      <c r="I327" t="n">
+        <v>100</v>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>heating and cooling company Birmingham AL</t>
+        </is>
+      </c>
+      <c r="K327" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L327" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>Western Sales and Services</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>westernsalesandservices.com</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>https://westernsalesandservices.com/</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>Air Conditioners</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>no-reply@westernsalesandservices.com</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>205-787-8674</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>Birmingham AL</t>
+        </is>
+      </c>
+      <c r="I328" t="n">
+        <v>100</v>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>heating and cooling company Birmingham AL</t>
+        </is>
+      </c>
+      <c r="K328" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L328" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 23:38 UTC (cycle 203)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L328"/>
+  <dimension ref="A1:L329"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -19578,6 +19578,66 @@
         </is>
       </c>
     </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>Pendergrass &amp; Holder Plumbing</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>pendergrassplumbing.com</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>https://pendergrassplumbing.com/residential/sewer-line-repair-winston-salem/</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>Line Service</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>service@pendergrassplumbing.com</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>(336) 924-1584</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="I329" t="n">
+        <v>90</v>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>sewer repair Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="K329" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L329" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 23:39 UTC (cycle 204)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L329"/>
+  <dimension ref="A1:L330"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -19638,6 +19638,62 @@
         </is>
       </c>
     </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>Sun Air Conditioning &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>sunairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>https://sunairconditioning.com/air-conditioning/ac-installation</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr"/>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>rusty@sunairconditioning.com</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>(281) 499-3916</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="I330" t="n">
+        <v>100</v>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>AC installation Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="K330" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L330" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>